<commit_message>
[HUMAN-VALIDATION]: Complited first sheet.
</commit_message>
<xml_diff>
--- a/thesis_evidence/validazione_umana/02_VALUTAZIONE_UMANA.xlsx
+++ b/thesis_evidence/validazione_umana/02_VALUTAZIONE_UMANA.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="Valutazioni" sheetId="1" state="visible" r:id="rId3"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2926" uniqueCount="1072">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2972" uniqueCount="1071">
   <si>
     <t xml:space="preserve">Valutazione delle 250 risposte del test</t>
   </si>
@@ -19362,9 +19362,6 @@
   </si>
   <si>
     <t xml:space="preserve">COMPLETO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DA COMPILARE</t>
   </si>
   <si>
     <t xml:space="preserve">Rubrica di valutazione</t>
@@ -20210,7 +20207,7 @@
       </c>
       <c r="B7" s="9" t="n">
         <f aca="false">COUNTIF(S9:S258,"OK")</f>
-        <v>40</v>
+        <v>50</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22594,18 +22591,34 @@
       <c r="I49" s="14" t="s">
         <v>243</v>
       </c>
-      <c r="J49" s="15"/>
-      <c r="K49" s="15"/>
-      <c r="L49" s="15"/>
-      <c r="M49" s="15"/>
-      <c r="N49" s="15"/>
-      <c r="O49" s="15"/>
-      <c r="P49" s="15"/>
-      <c r="Q49" s="15"/>
+      <c r="J49" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="K49" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L49" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M49" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N49" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O49" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="P49" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q49" s="15" t="s">
+        <v>36</v>
+      </c>
       <c r="R49" s="15"/>
       <c r="S49" s="16" t="str">
         <f aca="false">IF(AND(G49&lt;&gt;"",COUNT(J49:N49)=5,OR(ISNUMBER(O49),O49="N/A"),P49&lt;&gt;"",Q49&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22636,18 +22649,34 @@
       <c r="I50" s="14" t="s">
         <v>247</v>
       </c>
-      <c r="J50" s="15"/>
-      <c r="K50" s="15"/>
-      <c r="L50" s="15"/>
-      <c r="M50" s="15"/>
-      <c r="N50" s="15"/>
-      <c r="O50" s="15"/>
-      <c r="P50" s="15"/>
-      <c r="Q50" s="15"/>
+      <c r="J50" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="K50" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L50" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M50" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N50" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O50" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="P50" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q50" s="15" t="s">
+        <v>36</v>
+      </c>
       <c r="R50" s="15"/>
       <c r="S50" s="16" t="str">
         <f aca="false">IF(AND(G50&lt;&gt;"",COUNT(J50:N50)=5,OR(ISNUMBER(O50),O50="N/A"),P50&lt;&gt;"",Q50&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22674,18 +22703,34 @@
       </c>
       <c r="H51" s="14"/>
       <c r="I51" s="14"/>
-      <c r="J51" s="15"/>
-      <c r="K51" s="15"/>
-      <c r="L51" s="15"/>
-      <c r="M51" s="15"/>
-      <c r="N51" s="15"/>
-      <c r="O51" s="15"/>
-      <c r="P51" s="15"/>
-      <c r="Q51" s="15"/>
+      <c r="J51" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="K51" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L51" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M51" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N51" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O51" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="P51" s="15" t="s">
+        <v>95</v>
+      </c>
+      <c r="Q51" s="15" t="s">
+        <v>36</v>
+      </c>
       <c r="R51" s="15"/>
       <c r="S51" s="16" t="str">
         <f aca="false">IF(AND(G51&lt;&gt;"",COUNT(J51:N51)=5,OR(ISNUMBER(O51),O51="N/A"),P51&lt;&gt;"",Q51&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22712,18 +22757,34 @@
       </c>
       <c r="H52" s="14"/>
       <c r="I52" s="14"/>
-      <c r="J52" s="15"/>
-      <c r="K52" s="15"/>
-      <c r="L52" s="15"/>
-      <c r="M52" s="15"/>
-      <c r="N52" s="15"/>
-      <c r="O52" s="15"/>
-      <c r="P52" s="15"/>
-      <c r="Q52" s="15"/>
+      <c r="J52" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="K52" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L52" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M52" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N52" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="O52" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="P52" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q52" s="15" t="s">
+        <v>125</v>
+      </c>
       <c r="R52" s="15"/>
       <c r="S52" s="16" t="str">
         <f aca="false">IF(AND(G52&lt;&gt;"",COUNT(J52:N52)=5,OR(ISNUMBER(O52),O52="N/A"),P52&lt;&gt;"",Q52&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22754,18 +22815,34 @@
       <c r="I53" s="14" t="s">
         <v>258</v>
       </c>
-      <c r="J53" s="15"/>
-      <c r="K53" s="15"/>
-      <c r="L53" s="15"/>
-      <c r="M53" s="15"/>
-      <c r="N53" s="15"/>
-      <c r="O53" s="15"/>
-      <c r="P53" s="15"/>
-      <c r="Q53" s="15"/>
+      <c r="J53" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="K53" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L53" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M53" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N53" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O53" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="P53" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q53" s="15" t="s">
+        <v>36</v>
+      </c>
       <c r="R53" s="15"/>
       <c r="S53" s="16" t="str">
         <f aca="false">IF(AND(G53&lt;&gt;"",COUNT(J53:N53)=5,OR(ISNUMBER(O53),O53="N/A"),P53&lt;&gt;"",Q53&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22796,18 +22873,34 @@
       <c r="I54" s="14" t="s">
         <v>262</v>
       </c>
-      <c r="J54" s="15"/>
-      <c r="K54" s="15"/>
-      <c r="L54" s="15"/>
-      <c r="M54" s="15"/>
-      <c r="N54" s="15"/>
-      <c r="O54" s="15"/>
-      <c r="P54" s="15"/>
-      <c r="Q54" s="15"/>
+      <c r="J54" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="K54" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L54" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M54" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N54" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O54" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="P54" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q54" s="15" t="s">
+        <v>36</v>
+      </c>
       <c r="R54" s="15"/>
       <c r="S54" s="16" t="str">
         <f aca="false">IF(AND(G54&lt;&gt;"",COUNT(J54:N54)=5,OR(ISNUMBER(O54),O54="N/A"),P54&lt;&gt;"",Q54&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22838,18 +22931,34 @@
       <c r="I55" s="14" t="s">
         <v>268</v>
       </c>
-      <c r="J55" s="15"/>
-      <c r="K55" s="15"/>
-      <c r="L55" s="15"/>
-      <c r="M55" s="15"/>
-      <c r="N55" s="15"/>
-      <c r="O55" s="15"/>
-      <c r="P55" s="15"/>
-      <c r="Q55" s="15"/>
+      <c r="J55" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="K55" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L55" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M55" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N55" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O55" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="P55" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q55" s="15" t="s">
+        <v>36</v>
+      </c>
       <c r="R55" s="15"/>
       <c r="S55" s="16" t="str">
         <f aca="false">IF(AND(G55&lt;&gt;"",COUNT(J55:N55)=5,OR(ISNUMBER(O55),O55="N/A"),P55&lt;&gt;"",Q55&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22880,18 +22989,34 @@
       <c r="I56" s="14" t="s">
         <v>272</v>
       </c>
-      <c r="J56" s="15"/>
-      <c r="K56" s="15"/>
-      <c r="L56" s="15"/>
-      <c r="M56" s="15"/>
-      <c r="N56" s="15"/>
-      <c r="O56" s="15"/>
-      <c r="P56" s="15"/>
-      <c r="Q56" s="15"/>
+      <c r="J56" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="K56" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="L56" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M56" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N56" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O56" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="P56" s="15" t="s">
+        <v>95</v>
+      </c>
+      <c r="Q56" s="15" t="s">
+        <v>75</v>
+      </c>
       <c r="R56" s="15"/>
       <c r="S56" s="16" t="str">
         <f aca="false">IF(AND(G56&lt;&gt;"",COUNT(J56:N56)=5,OR(ISNUMBER(O56),O56="N/A"),P56&lt;&gt;"",Q56&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22922,18 +23047,34 @@
       <c r="I57" s="14" t="s">
         <v>278</v>
       </c>
-      <c r="J57" s="15"/>
-      <c r="K57" s="15"/>
-      <c r="L57" s="15"/>
-      <c r="M57" s="15"/>
-      <c r="N57" s="15"/>
-      <c r="O57" s="15"/>
-      <c r="P57" s="15"/>
-      <c r="Q57" s="15"/>
+      <c r="J57" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="K57" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L57" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M57" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N57" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O57" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="P57" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q57" s="15" t="s">
+        <v>36</v>
+      </c>
       <c r="R57" s="15"/>
       <c r="S57" s="16" t="str">
         <f aca="false">IF(AND(G57&lt;&gt;"",COUNT(J57:N57)=5,OR(ISNUMBER(O57),O57="N/A"),P57&lt;&gt;"",Q57&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22964,18 +23105,34 @@
       <c r="I58" s="14" t="s">
         <v>282</v>
       </c>
-      <c r="J58" s="15"/>
-      <c r="K58" s="15"/>
-      <c r="L58" s="15"/>
-      <c r="M58" s="15"/>
-      <c r="N58" s="15"/>
-      <c r="O58" s="15"/>
-      <c r="P58" s="15"/>
-      <c r="Q58" s="15"/>
+      <c r="J58" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="K58" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L58" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M58" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N58" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O58" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="P58" s="15" t="s">
+        <v>95</v>
+      </c>
+      <c r="Q58" s="15" t="s">
+        <v>36</v>
+      </c>
       <c r="R58" s="15"/>
       <c r="S58" s="16" t="str">
         <f aca="false">IF(AND(G58&lt;&gt;"",COUNT(J58:N58)=5,OR(ISNUMBER(O58),O58="N/A"),P58&lt;&gt;"",Q58&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -31362,7 +31519,7 @@
         <v>50</v>
       </c>
       <c r="C6" s="1" t="n">
-        <v>40</v>
+        <v>50</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -33708,17 +33865,33 @@
       <c r="I48" s="14" t="s">
         <v>846</v>
       </c>
-      <c r="J48" s="15"/>
-      <c r="K48" s="15"/>
-      <c r="L48" s="15"/>
-      <c r="M48" s="15"/>
-      <c r="N48" s="15"/>
-      <c r="O48" s="15"/>
-      <c r="P48" s="15"/>
-      <c r="Q48" s="15"/>
+      <c r="J48" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="K48" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L48" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M48" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N48" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O48" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="P48" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q48" s="15" t="s">
+        <v>36</v>
+      </c>
       <c r="R48" s="15"/>
       <c r="S48" s="13" t="s">
-        <v>1022</v>
+        <v>1021</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -33749,17 +33922,33 @@
       <c r="I49" s="14" t="s">
         <v>849</v>
       </c>
-      <c r="J49" s="15"/>
-      <c r="K49" s="15"/>
-      <c r="L49" s="15"/>
-      <c r="M49" s="15"/>
-      <c r="N49" s="15"/>
-      <c r="O49" s="15"/>
-      <c r="P49" s="15"/>
-      <c r="Q49" s="15"/>
+      <c r="J49" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="K49" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L49" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M49" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N49" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O49" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="P49" s="15" t="s">
+        <v>95</v>
+      </c>
+      <c r="Q49" s="15" t="s">
+        <v>75</v>
+      </c>
       <c r="R49" s="15"/>
       <c r="S49" s="13" t="s">
-        <v>1022</v>
+        <v>1021</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -33790,17 +33979,33 @@
       <c r="I50" s="14" t="s">
         <v>885</v>
       </c>
-      <c r="J50" s="15"/>
-      <c r="K50" s="15"/>
-      <c r="L50" s="15"/>
-      <c r="M50" s="15"/>
-      <c r="N50" s="15"/>
-      <c r="O50" s="15"/>
-      <c r="P50" s="15"/>
-      <c r="Q50" s="15"/>
+      <c r="J50" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="K50" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L50" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M50" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N50" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O50" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="P50" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q50" s="15" t="s">
+        <v>75</v>
+      </c>
       <c r="R50" s="15"/>
       <c r="S50" s="13" t="s">
-        <v>1022</v>
+        <v>1021</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -33827,17 +34032,33 @@
       </c>
       <c r="H51" s="14"/>
       <c r="I51" s="14"/>
-      <c r="J51" s="15"/>
-      <c r="K51" s="15"/>
-      <c r="L51" s="15"/>
-      <c r="M51" s="15"/>
-      <c r="N51" s="15"/>
-      <c r="O51" s="15"/>
-      <c r="P51" s="15"/>
-      <c r="Q51" s="15"/>
+      <c r="J51" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="K51" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L51" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M51" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N51" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O51" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="P51" s="15" t="s">
+        <v>95</v>
+      </c>
+      <c r="Q51" s="15" t="s">
+        <v>36</v>
+      </c>
       <c r="R51" s="15"/>
       <c r="S51" s="13" t="s">
-        <v>1022</v>
+        <v>1021</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -33868,17 +34089,33 @@
       <c r="I52" s="14" t="s">
         <v>905</v>
       </c>
-      <c r="J52" s="15"/>
-      <c r="K52" s="15"/>
-      <c r="L52" s="15"/>
-      <c r="M52" s="15"/>
-      <c r="N52" s="15"/>
-      <c r="O52" s="15"/>
-      <c r="P52" s="15"/>
-      <c r="Q52" s="15"/>
+      <c r="J52" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="K52" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L52" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M52" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N52" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O52" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="P52" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q52" s="15" t="s">
+        <v>36</v>
+      </c>
       <c r="R52" s="15"/>
       <c r="S52" s="13" t="s">
-        <v>1022</v>
+        <v>1021</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -33905,17 +34142,33 @@
       </c>
       <c r="H53" s="14"/>
       <c r="I53" s="14"/>
-      <c r="J53" s="15"/>
-      <c r="K53" s="15"/>
-      <c r="L53" s="15"/>
-      <c r="M53" s="15"/>
-      <c r="N53" s="15"/>
-      <c r="O53" s="15"/>
-      <c r="P53" s="15"/>
-      <c r="Q53" s="15"/>
+      <c r="J53" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="K53" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L53" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M53" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N53" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O53" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="P53" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q53" s="15" t="s">
+        <v>125</v>
+      </c>
       <c r="R53" s="15"/>
       <c r="S53" s="13" t="s">
-        <v>1022</v>
+        <v>1021</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -33946,17 +34199,33 @@
       <c r="I54" s="14" t="s">
         <v>911</v>
       </c>
-      <c r="J54" s="15"/>
-      <c r="K54" s="15"/>
-      <c r="L54" s="15"/>
-      <c r="M54" s="15"/>
-      <c r="N54" s="15"/>
-      <c r="O54" s="15"/>
-      <c r="P54" s="15"/>
-      <c r="Q54" s="15"/>
+      <c r="J54" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="K54" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L54" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M54" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N54" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O54" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="P54" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q54" s="15" t="s">
+        <v>36</v>
+      </c>
       <c r="R54" s="15"/>
       <c r="S54" s="13" t="s">
-        <v>1022</v>
+        <v>1021</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -33987,17 +34256,33 @@
       <c r="I55" s="14" t="s">
         <v>940</v>
       </c>
-      <c r="J55" s="15"/>
-      <c r="K55" s="15"/>
-      <c r="L55" s="15"/>
-      <c r="M55" s="15"/>
-      <c r="N55" s="15"/>
-      <c r="O55" s="15"/>
-      <c r="P55" s="15"/>
-      <c r="Q55" s="15"/>
+      <c r="J55" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="K55" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L55" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M55" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N55" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O55" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="P55" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q55" s="15" t="s">
+        <v>36</v>
+      </c>
       <c r="R55" s="15"/>
       <c r="S55" s="13" t="s">
-        <v>1022</v>
+        <v>1021</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -34024,17 +34309,33 @@
       </c>
       <c r="H56" s="14"/>
       <c r="I56" s="14"/>
-      <c r="J56" s="15"/>
-      <c r="K56" s="15"/>
-      <c r="L56" s="15"/>
-      <c r="M56" s="15"/>
-      <c r="N56" s="15"/>
-      <c r="O56" s="15"/>
-      <c r="P56" s="15"/>
-      <c r="Q56" s="15"/>
+      <c r="J56" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="K56" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L56" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M56" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N56" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O56" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="P56" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q56" s="15" t="s">
+        <v>125</v>
+      </c>
       <c r="R56" s="15"/>
       <c r="S56" s="13" t="s">
-        <v>1022</v>
+        <v>1021</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -34061,17 +34362,33 @@
       </c>
       <c r="H57" s="14"/>
       <c r="I57" s="14"/>
-      <c r="J57" s="15"/>
-      <c r="K57" s="15"/>
-      <c r="L57" s="15"/>
-      <c r="M57" s="15"/>
-      <c r="N57" s="15"/>
-      <c r="O57" s="15"/>
-      <c r="P57" s="15"/>
-      <c r="Q57" s="15"/>
+      <c r="J57" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="K57" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L57" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M57" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N57" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O57" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="P57" s="15" t="s">
+        <v>95</v>
+      </c>
+      <c r="Q57" s="15" t="s">
+        <v>36</v>
+      </c>
       <c r="R57" s="15"/>
       <c r="S57" s="13" t="s">
-        <v>1022</v>
+        <v>1021</v>
       </c>
     </row>
     <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
@@ -34148,292 +34465,292 @@
   <sheetData>
     <row r="2" customFormat="false" ht="25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>1023</v>
+        <v>1022</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
     </row>
     <row r="4" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="10" t="s">
+        <v>1023</v>
+      </c>
+      <c r="B4" s="10" t="s">
         <v>1024</v>
       </c>
-      <c r="B4" s="10" t="s">
+      <c r="C4" s="10" t="s">
         <v>1025</v>
-      </c>
-      <c r="C4" s="10" t="s">
-        <v>1026</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="19" t="s">
-        <v>1027</v>
+        <v>1026</v>
       </c>
       <c r="B5" s="20" t="n">
         <v>0</v>
       </c>
       <c r="C5" s="19" t="s">
-        <v>1028</v>
+        <v>1027</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="21" t="s">
-        <v>1027</v>
+        <v>1026</v>
       </c>
       <c r="B6" s="22" t="n">
         <v>1</v>
       </c>
       <c r="C6" s="21" t="s">
-        <v>1029</v>
+        <v>1028</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="21" t="s">
-        <v>1027</v>
+        <v>1026</v>
       </c>
       <c r="B7" s="22" t="n">
         <v>2</v>
       </c>
       <c r="C7" s="21" t="s">
-        <v>1030</v>
+        <v>1029</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="21" t="s">
-        <v>1027</v>
+        <v>1026</v>
       </c>
       <c r="B8" s="22" t="n">
         <v>3</v>
       </c>
       <c r="C8" s="21" t="s">
-        <v>1031</v>
+        <v>1030</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="21" t="s">
-        <v>1032</v>
+        <v>1031</v>
       </c>
       <c r="B9" s="22" t="n">
         <v>0</v>
       </c>
       <c r="C9" s="21" t="s">
-        <v>1033</v>
+        <v>1032</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="21" t="s">
-        <v>1032</v>
+        <v>1031</v>
       </c>
       <c r="B10" s="22" t="n">
         <v>1</v>
       </c>
       <c r="C10" s="21" t="s">
-        <v>1034</v>
+        <v>1033</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="21" t="s">
-        <v>1032</v>
+        <v>1031</v>
       </c>
       <c r="B11" s="22" t="n">
         <v>2</v>
       </c>
       <c r="C11" s="21" t="s">
-        <v>1035</v>
+        <v>1034</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="21" t="s">
-        <v>1032</v>
+        <v>1031</v>
       </c>
       <c r="B12" s="22" t="n">
         <v>3</v>
       </c>
       <c r="C12" s="21" t="s">
-        <v>1036</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="21" t="s">
-        <v>1037</v>
+        <v>1036</v>
       </c>
       <c r="B13" s="22" t="n">
         <v>0</v>
       </c>
       <c r="C13" s="21" t="s">
-        <v>1038</v>
+        <v>1037</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="21" t="s">
-        <v>1037</v>
+        <v>1036</v>
       </c>
       <c r="B14" s="22" t="n">
         <v>1</v>
       </c>
       <c r="C14" s="21" t="s">
-        <v>1039</v>
+        <v>1038</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="21" t="s">
-        <v>1037</v>
+        <v>1036</v>
       </c>
       <c r="B15" s="22" t="n">
         <v>2</v>
       </c>
       <c r="C15" s="21" t="s">
-        <v>1040</v>
+        <v>1039</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="21" t="s">
-        <v>1037</v>
+        <v>1036</v>
       </c>
       <c r="B16" s="22" t="n">
         <v>3</v>
       </c>
       <c r="C16" s="21" t="s">
-        <v>1041</v>
+        <v>1040</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="21" t="s">
-        <v>1042</v>
+        <v>1041</v>
       </c>
       <c r="B17" s="22" t="n">
         <v>0</v>
       </c>
       <c r="C17" s="21" t="s">
-        <v>1043</v>
+        <v>1042</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="21" t="s">
-        <v>1042</v>
+        <v>1041</v>
       </c>
       <c r="B18" s="22" t="n">
         <v>1</v>
       </c>
       <c r="C18" s="21" t="s">
-        <v>1044</v>
+        <v>1043</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="21" t="s">
-        <v>1042</v>
+        <v>1041</v>
       </c>
       <c r="B19" s="22" t="n">
         <v>2</v>
       </c>
       <c r="C19" s="21" t="s">
-        <v>1045</v>
+        <v>1044</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="21" t="s">
-        <v>1042</v>
+        <v>1041</v>
       </c>
       <c r="B20" s="22" t="n">
         <v>3</v>
       </c>
       <c r="C20" s="21" t="s">
-        <v>1046</v>
+        <v>1045</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="21" t="s">
-        <v>1047</v>
+        <v>1046</v>
       </c>
       <c r="B21" s="22" t="n">
         <v>0</v>
       </c>
       <c r="C21" s="21" t="s">
-        <v>1048</v>
+        <v>1047</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="21" t="s">
-        <v>1047</v>
+        <v>1046</v>
       </c>
       <c r="B22" s="22" t="n">
         <v>1</v>
       </c>
       <c r="C22" s="21" t="s">
-        <v>1049</v>
+        <v>1048</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="21" t="s">
-        <v>1047</v>
+        <v>1046</v>
       </c>
       <c r="B23" s="22" t="n">
         <v>2</v>
       </c>
       <c r="C23" s="21" t="s">
-        <v>1050</v>
+        <v>1049</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="21" t="s">
-        <v>1047</v>
+        <v>1046</v>
       </c>
       <c r="B24" s="22" t="n">
         <v>3</v>
       </c>
       <c r="C24" s="21" t="s">
-        <v>1051</v>
+        <v>1050</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="21" t="s">
-        <v>1052</v>
+        <v>1051</v>
       </c>
       <c r="B25" s="22" t="n">
         <v>0</v>
       </c>
       <c r="C25" s="21" t="s">
-        <v>1053</v>
+        <v>1052</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="21" t="s">
-        <v>1052</v>
+        <v>1051</v>
       </c>
       <c r="B26" s="22" t="n">
         <v>1</v>
       </c>
       <c r="C26" s="21" t="s">
-        <v>1054</v>
+        <v>1053</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="21" t="s">
-        <v>1052</v>
+        <v>1051</v>
       </c>
       <c r="B27" s="22" t="n">
         <v>2</v>
       </c>
       <c r="C27" s="21" t="s">
-        <v>1055</v>
+        <v>1054</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="21" t="s">
-        <v>1052</v>
+        <v>1051</v>
       </c>
       <c r="B28" s="22" t="n">
         <v>3</v>
       </c>
       <c r="C28" s="21" t="s">
-        <v>1056</v>
+        <v>1055</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="10" t="s">
+        <v>1056</v>
+      </c>
+      <c r="B31" s="10" t="s">
         <v>1057</v>
-      </c>
-      <c r="B31" s="10" t="s">
-        <v>1058</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -34441,7 +34758,7 @@
         <v>35</v>
       </c>
       <c r="B32" s="19" t="s">
-        <v>1059</v>
+        <v>1058</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -34449,7 +34766,7 @@
         <v>95</v>
       </c>
       <c r="B33" s="21" t="s">
-        <v>1060</v>
+        <v>1059</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -34457,7 +34774,7 @@
         <v>116</v>
       </c>
       <c r="B34" s="21" t="s">
-        <v>1061</v>
+        <v>1060</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -34465,47 +34782,47 @@
         <v>74</v>
       </c>
       <c r="B35" s="21" t="s">
-        <v>1062</v>
+        <v>1061</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="10" t="s">
-        <v>1063</v>
+        <v>1062</v>
       </c>
       <c r="B37" s="10" t="s">
-        <v>1058</v>
+        <v>1057</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="19" t="s">
+        <v>1063</v>
+      </c>
+      <c r="B38" s="19" t="s">
         <v>1064</v>
-      </c>
-      <c r="B38" s="19" t="s">
-        <v>1065</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="21" t="s">
+        <v>1065</v>
+      </c>
+      <c r="B39" s="21" t="s">
         <v>1066</v>
-      </c>
-      <c r="B39" s="21" t="s">
-        <v>1067</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="21" t="s">
+        <v>1067</v>
+      </c>
+      <c r="B40" s="21" t="s">
         <v>1068</v>
-      </c>
-      <c r="B40" s="21" t="s">
-        <v>1069</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="21" t="s">
+        <v>1069</v>
+      </c>
+      <c r="B41" s="21" t="s">
         <v>1070</v>
-      </c>
-      <c r="B41" s="21" t="s">
-        <v>1071</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
[HUMAN-VALIDATION]: Increased validated cases.
</commit_message>
<xml_diff>
--- a/thesis_evidence/validazione_umana/02_VALUTAZIONE_UMANA.xlsx
+++ b/thesis_evidence/validazione_umana/02_VALUTAZIONE_UMANA.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2972" uniqueCount="1071">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3025" uniqueCount="1071">
   <si>
     <t xml:space="preserve">Valutazione delle 250 risposte del test</t>
   </si>
@@ -20207,7 +20207,7 @@
       </c>
       <c r="B7" s="9" t="n">
         <f aca="false">COUNTIF(S9:S258,"OK")</f>
-        <v>50</v>
+        <v>73</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23159,18 +23159,34 @@
       </c>
       <c r="H59" s="14"/>
       <c r="I59" s="14"/>
-      <c r="J59" s="15"/>
-      <c r="K59" s="15"/>
-      <c r="L59" s="15"/>
-      <c r="M59" s="15"/>
-      <c r="N59" s="15"/>
-      <c r="O59" s="15"/>
-      <c r="P59" s="15"/>
-      <c r="Q59" s="15"/>
+      <c r="J59" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="K59" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L59" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M59" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N59" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O59" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="P59" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q59" s="15" t="s">
+        <v>36</v>
+      </c>
       <c r="R59" s="15"/>
       <c r="S59" s="16" t="str">
         <f aca="false">IF(AND(G59&lt;&gt;"",COUNT(J59:N59)=5,OR(ISNUMBER(O59),O59="N/A"),P59&lt;&gt;"",Q59&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23197,18 +23213,34 @@
       </c>
       <c r="H60" s="14"/>
       <c r="I60" s="14"/>
-      <c r="J60" s="15"/>
-      <c r="K60" s="15"/>
-      <c r="L60" s="15"/>
-      <c r="M60" s="15"/>
-      <c r="N60" s="15"/>
-      <c r="O60" s="15"/>
-      <c r="P60" s="15"/>
-      <c r="Q60" s="15"/>
+      <c r="J60" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="K60" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L60" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M60" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N60" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O60" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="P60" s="15" t="s">
+        <v>95</v>
+      </c>
+      <c r="Q60" s="15" t="s">
+        <v>36</v>
+      </c>
       <c r="R60" s="15"/>
       <c r="S60" s="16" t="str">
         <f aca="false">IF(AND(G60&lt;&gt;"",COUNT(J60:N60)=5,OR(ISNUMBER(O60),O60="N/A"),P60&lt;&gt;"",Q60&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23239,18 +23271,34 @@
       <c r="I61" s="14" t="s">
         <v>293</v>
       </c>
-      <c r="J61" s="15"/>
-      <c r="K61" s="15"/>
-      <c r="L61" s="15"/>
-      <c r="M61" s="15"/>
-      <c r="N61" s="15"/>
-      <c r="O61" s="15"/>
-      <c r="P61" s="15"/>
-      <c r="Q61" s="15"/>
+      <c r="J61" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="K61" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L61" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M61" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N61" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O61" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="P61" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q61" s="15" t="s">
+        <v>36</v>
+      </c>
       <c r="R61" s="15"/>
       <c r="S61" s="16" t="str">
         <f aca="false">IF(AND(G61&lt;&gt;"",COUNT(J61:N61)=5,OR(ISNUMBER(O61),O61="N/A"),P61&lt;&gt;"",Q61&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23281,18 +23329,34 @@
       <c r="I62" s="14" t="s">
         <v>297</v>
       </c>
-      <c r="J62" s="15"/>
-      <c r="K62" s="15"/>
-      <c r="L62" s="15"/>
-      <c r="M62" s="15"/>
-      <c r="N62" s="15"/>
-      <c r="O62" s="15"/>
-      <c r="P62" s="15"/>
-      <c r="Q62" s="15"/>
+      <c r="J62" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="K62" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L62" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M62" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N62" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O62" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="P62" s="15" t="s">
+        <v>95</v>
+      </c>
+      <c r="Q62" s="15" t="s">
+        <v>36</v>
+      </c>
       <c r="R62" s="15"/>
       <c r="S62" s="16" t="str">
         <f aca="false">IF(AND(G62&lt;&gt;"",COUNT(J62:N62)=5,OR(ISNUMBER(O62),O62="N/A"),P62&lt;&gt;"",Q62&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23323,18 +23387,34 @@
       <c r="I63" s="14" t="s">
         <v>301</v>
       </c>
-      <c r="J63" s="15"/>
-      <c r="K63" s="15"/>
-      <c r="L63" s="15"/>
-      <c r="M63" s="15"/>
-      <c r="N63" s="15"/>
-      <c r="O63" s="15"/>
-      <c r="P63" s="15"/>
-      <c r="Q63" s="15"/>
+      <c r="J63" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="K63" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L63" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M63" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N63" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O63" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="P63" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q63" s="15" t="s">
+        <v>36</v>
+      </c>
       <c r="R63" s="15"/>
       <c r="S63" s="16" t="str">
         <f aca="false">IF(AND(G63&lt;&gt;"",COUNT(J63:N63)=5,OR(ISNUMBER(O63),O63="N/A"),P63&lt;&gt;"",Q63&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23365,18 +23445,34 @@
       <c r="I64" s="14" t="s">
         <v>304</v>
       </c>
-      <c r="J64" s="15"/>
-      <c r="K64" s="15"/>
-      <c r="L64" s="15"/>
-      <c r="M64" s="15"/>
-      <c r="N64" s="15"/>
-      <c r="O64" s="15"/>
-      <c r="P64" s="15"/>
-      <c r="Q64" s="15"/>
+      <c r="J64" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="K64" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="L64" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M64" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N64" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O64" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="P64" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q64" s="15" t="s">
+        <v>75</v>
+      </c>
       <c r="R64" s="15"/>
       <c r="S64" s="16" t="str">
         <f aca="false">IF(AND(G64&lt;&gt;"",COUNT(J64:N64)=5,OR(ISNUMBER(O64),O64="N/A"),P64&lt;&gt;"",Q64&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23407,18 +23503,34 @@
       <c r="I65" s="14" t="s">
         <v>310</v>
       </c>
-      <c r="J65" s="15"/>
-      <c r="K65" s="15"/>
-      <c r="L65" s="15"/>
-      <c r="M65" s="15"/>
-      <c r="N65" s="15"/>
-      <c r="O65" s="15"/>
-      <c r="P65" s="15"/>
-      <c r="Q65" s="15"/>
+      <c r="J65" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="K65" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L65" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M65" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N65" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O65" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="P65" s="15" t="s">
+        <v>95</v>
+      </c>
+      <c r="Q65" s="15" t="s">
+        <v>36</v>
+      </c>
       <c r="R65" s="15"/>
       <c r="S65" s="16" t="str">
         <f aca="false">IF(AND(G65&lt;&gt;"",COUNT(J65:N65)=5,OR(ISNUMBER(O65),O65="N/A"),P65&lt;&gt;"",Q65&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23449,18 +23561,34 @@
       <c r="I66" s="14" t="s">
         <v>314</v>
       </c>
-      <c r="J66" s="15"/>
-      <c r="K66" s="15"/>
-      <c r="L66" s="15"/>
-      <c r="M66" s="15"/>
-      <c r="N66" s="15"/>
-      <c r="O66" s="15"/>
-      <c r="P66" s="15"/>
-      <c r="Q66" s="15"/>
+      <c r="J66" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="K66" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L66" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M66" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N66" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O66" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="P66" s="15" t="s">
+        <v>95</v>
+      </c>
+      <c r="Q66" s="15" t="s">
+        <v>75</v>
+      </c>
       <c r="R66" s="15"/>
       <c r="S66" s="16" t="str">
         <f aca="false">IF(AND(G66&lt;&gt;"",COUNT(J66:N66)=5,OR(ISNUMBER(O66),O66="N/A"),P66&lt;&gt;"",Q66&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23487,18 +23615,34 @@
       </c>
       <c r="H67" s="14"/>
       <c r="I67" s="14"/>
-      <c r="J67" s="15"/>
-      <c r="K67" s="15"/>
-      <c r="L67" s="15"/>
-      <c r="M67" s="15"/>
-      <c r="N67" s="15"/>
-      <c r="O67" s="15"/>
-      <c r="P67" s="15"/>
-      <c r="Q67" s="15"/>
+      <c r="J67" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="K67" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L67" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M67" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N67" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O67" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="P67" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q67" s="15" t="s">
+        <v>36</v>
+      </c>
       <c r="R67" s="15"/>
       <c r="S67" s="16" t="str">
         <f aca="false">IF(AND(G67&lt;&gt;"",COUNT(J67:N67)=5,OR(ISNUMBER(O67),O67="N/A"),P67&lt;&gt;"",Q67&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23529,18 +23673,34 @@
       <c r="I68" s="14" t="s">
         <v>320</v>
       </c>
-      <c r="J68" s="15"/>
-      <c r="K68" s="15"/>
-      <c r="L68" s="15"/>
-      <c r="M68" s="15"/>
-      <c r="N68" s="15"/>
-      <c r="O68" s="15"/>
-      <c r="P68" s="15"/>
-      <c r="Q68" s="15"/>
+      <c r="J68" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="K68" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L68" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M68" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N68" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O68" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="P68" s="15" t="s">
+        <v>95</v>
+      </c>
+      <c r="Q68" s="15" t="s">
+        <v>36</v>
+      </c>
       <c r="R68" s="15"/>
       <c r="S68" s="16" t="str">
         <f aca="false">IF(AND(G68&lt;&gt;"",COUNT(J68:N68)=5,OR(ISNUMBER(O68),O68="N/A"),P68&lt;&gt;"",Q68&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23571,18 +23731,34 @@
       <c r="I69" s="14" t="s">
         <v>325</v>
       </c>
-      <c r="J69" s="15"/>
-      <c r="K69" s="15"/>
-      <c r="L69" s="15"/>
-      <c r="M69" s="15"/>
-      <c r="N69" s="15"/>
-      <c r="O69" s="15"/>
-      <c r="P69" s="15"/>
-      <c r="Q69" s="15"/>
+      <c r="J69" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="K69" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L69" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M69" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N69" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O69" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="P69" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q69" s="15" t="s">
+        <v>75</v>
+      </c>
       <c r="R69" s="15"/>
       <c r="S69" s="16" t="str">
         <f aca="false">IF(AND(G69&lt;&gt;"",COUNT(J69:N69)=5,OR(ISNUMBER(O69),O69="N/A"),P69&lt;&gt;"",Q69&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23613,18 +23789,34 @@
       <c r="I70" s="14" t="s">
         <v>329</v>
       </c>
-      <c r="J70" s="15"/>
-      <c r="K70" s="15"/>
-      <c r="L70" s="15"/>
-      <c r="M70" s="15"/>
-      <c r="N70" s="15"/>
-      <c r="O70" s="15"/>
-      <c r="P70" s="15"/>
-      <c r="Q70" s="15"/>
+      <c r="J70" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="K70" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L70" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M70" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N70" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O70" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="P70" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q70" s="15" t="s">
+        <v>75</v>
+      </c>
       <c r="R70" s="15"/>
       <c r="S70" s="16" t="str">
         <f aca="false">IF(AND(G70&lt;&gt;"",COUNT(J70:N70)=5,OR(ISNUMBER(O70),O70="N/A"),P70&lt;&gt;"",Q70&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23655,18 +23847,34 @@
       <c r="I71" s="14" t="s">
         <v>333</v>
       </c>
-      <c r="J71" s="15"/>
-      <c r="K71" s="15"/>
-      <c r="L71" s="15"/>
-      <c r="M71" s="15"/>
-      <c r="N71" s="15"/>
-      <c r="O71" s="15"/>
-      <c r="P71" s="15"/>
-      <c r="Q71" s="15"/>
+      <c r="J71" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="K71" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L71" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M71" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N71" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O71" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="P71" s="15" t="s">
+        <v>74</v>
+      </c>
+      <c r="Q71" s="15" t="s">
+        <v>75</v>
+      </c>
       <c r="R71" s="15"/>
       <c r="S71" s="16" t="str">
         <f aca="false">IF(AND(G71&lt;&gt;"",COUNT(J71:N71)=5,OR(ISNUMBER(O71),O71="N/A"),P71&lt;&gt;"",Q71&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23697,18 +23905,34 @@
       <c r="I72" s="14" t="s">
         <v>338</v>
       </c>
-      <c r="J72" s="15"/>
-      <c r="K72" s="15"/>
-      <c r="L72" s="15"/>
-      <c r="M72" s="15"/>
-      <c r="N72" s="15"/>
-      <c r="O72" s="15"/>
-      <c r="P72" s="15"/>
-      <c r="Q72" s="15"/>
+      <c r="J72" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="K72" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L72" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M72" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N72" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O72" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="P72" s="15" t="s">
+        <v>95</v>
+      </c>
+      <c r="Q72" s="15" t="s">
+        <v>36</v>
+      </c>
       <c r="R72" s="15"/>
       <c r="S72" s="16" t="str">
         <f aca="false">IF(AND(G72&lt;&gt;"",COUNT(J72:N72)=5,OR(ISNUMBER(O72),O72="N/A"),P72&lt;&gt;"",Q72&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23735,18 +23959,34 @@
       </c>
       <c r="H73" s="14"/>
       <c r="I73" s="14"/>
-      <c r="J73" s="15"/>
-      <c r="K73" s="15"/>
-      <c r="L73" s="15"/>
-      <c r="M73" s="15"/>
-      <c r="N73" s="15"/>
-      <c r="O73" s="15"/>
-      <c r="P73" s="15"/>
-      <c r="Q73" s="15"/>
+      <c r="J73" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="K73" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L73" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M73" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N73" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O73" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="P73" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q73" s="15" t="s">
+        <v>36</v>
+      </c>
       <c r="R73" s="15"/>
       <c r="S73" s="16" t="str">
         <f aca="false">IF(AND(G73&lt;&gt;"",COUNT(J73:N73)=5,OR(ISNUMBER(O73),O73="N/A"),P73&lt;&gt;"",Q73&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23773,18 +24013,34 @@
       </c>
       <c r="H74" s="14"/>
       <c r="I74" s="14"/>
-      <c r="J74" s="15"/>
-      <c r="K74" s="15"/>
-      <c r="L74" s="15"/>
-      <c r="M74" s="15"/>
-      <c r="N74" s="15"/>
-      <c r="O74" s="15"/>
-      <c r="P74" s="15"/>
-      <c r="Q74" s="15"/>
+      <c r="J74" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="K74" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L74" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M74" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N74" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O74" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="P74" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q74" s="15" t="s">
+        <v>125</v>
+      </c>
       <c r="R74" s="15"/>
       <c r="S74" s="16" t="str">
         <f aca="false">IF(AND(G74&lt;&gt;"",COUNT(J74:N74)=5,OR(ISNUMBER(O74),O74="N/A"),P74&lt;&gt;"",Q74&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23811,18 +24067,34 @@
       </c>
       <c r="H75" s="14"/>
       <c r="I75" s="14"/>
-      <c r="J75" s="15"/>
-      <c r="K75" s="15"/>
-      <c r="L75" s="15"/>
-      <c r="M75" s="15"/>
-      <c r="N75" s="15"/>
-      <c r="O75" s="15"/>
-      <c r="P75" s="15"/>
-      <c r="Q75" s="15"/>
+      <c r="J75" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="K75" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L75" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M75" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N75" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O75" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="P75" s="15" t="s">
+        <v>74</v>
+      </c>
+      <c r="Q75" s="15" t="s">
+        <v>125</v>
+      </c>
       <c r="R75" s="15"/>
       <c r="S75" s="16" t="str">
         <f aca="false">IF(AND(G75&lt;&gt;"",COUNT(J75:N75)=5,OR(ISNUMBER(O75),O75="N/A"),P75&lt;&gt;"",Q75&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23853,18 +24125,34 @@
       <c r="I76" s="14" t="s">
         <v>348</v>
       </c>
-      <c r="J76" s="15"/>
-      <c r="K76" s="15"/>
-      <c r="L76" s="15"/>
-      <c r="M76" s="15"/>
-      <c r="N76" s="15"/>
-      <c r="O76" s="15"/>
-      <c r="P76" s="15"/>
-      <c r="Q76" s="15"/>
+      <c r="J76" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="K76" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L76" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M76" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N76" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O76" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="P76" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q76" s="15" t="s">
+        <v>36</v>
+      </c>
       <c r="R76" s="15"/>
       <c r="S76" s="16" t="str">
         <f aca="false">IF(AND(G76&lt;&gt;"",COUNT(J76:N76)=5,OR(ISNUMBER(O76),O76="N/A"),P76&lt;&gt;"",Q76&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23895,18 +24183,34 @@
       <c r="I77" s="14" t="s">
         <v>352</v>
       </c>
-      <c r="J77" s="15"/>
-      <c r="K77" s="15"/>
-      <c r="L77" s="15"/>
-      <c r="M77" s="15"/>
-      <c r="N77" s="15"/>
-      <c r="O77" s="15"/>
-      <c r="P77" s="15"/>
-      <c r="Q77" s="15"/>
+      <c r="J77" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="K77" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L77" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M77" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N77" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O77" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="P77" s="15" t="s">
+        <v>116</v>
+      </c>
+      <c r="Q77" s="15" t="s">
+        <v>117</v>
+      </c>
       <c r="R77" s="15"/>
       <c r="S77" s="16" t="str">
         <f aca="false">IF(AND(G77&lt;&gt;"",COUNT(J77:N77)=5,OR(ISNUMBER(O77),O77="N/A"),P77&lt;&gt;"",Q77&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23937,18 +24241,34 @@
       <c r="I78" s="14" t="s">
         <v>358</v>
       </c>
-      <c r="J78" s="15"/>
-      <c r="K78" s="15"/>
-      <c r="L78" s="15"/>
-      <c r="M78" s="15"/>
-      <c r="N78" s="15"/>
-      <c r="O78" s="15"/>
-      <c r="P78" s="15"/>
-      <c r="Q78" s="15"/>
+      <c r="J78" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="K78" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L78" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M78" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N78" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O78" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="P78" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q78" s="15" t="s">
+        <v>36</v>
+      </c>
       <c r="R78" s="15"/>
       <c r="S78" s="16" t="str">
         <f aca="false">IF(AND(G78&lt;&gt;"",COUNT(J78:N78)=5,OR(ISNUMBER(O78),O78="N/A"),P78&lt;&gt;"",Q78&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23975,18 +24295,34 @@
       </c>
       <c r="H79" s="14"/>
       <c r="I79" s="14"/>
-      <c r="J79" s="15"/>
-      <c r="K79" s="15"/>
-      <c r="L79" s="15"/>
-      <c r="M79" s="15"/>
-      <c r="N79" s="15"/>
-      <c r="O79" s="15"/>
-      <c r="P79" s="15"/>
-      <c r="Q79" s="15"/>
+      <c r="J79" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="K79" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L79" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M79" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N79" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O79" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="P79" s="15" t="s">
+        <v>95</v>
+      </c>
+      <c r="Q79" s="15" t="s">
+        <v>36</v>
+      </c>
       <c r="R79" s="15"/>
       <c r="S79" s="16" t="str">
         <f aca="false">IF(AND(G79&lt;&gt;"",COUNT(J79:N79)=5,OR(ISNUMBER(O79),O79="N/A"),P79&lt;&gt;"",Q79&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -24017,18 +24353,34 @@
       <c r="I80" s="14" t="s">
         <v>368</v>
       </c>
-      <c r="J80" s="15"/>
-      <c r="K80" s="15"/>
-      <c r="L80" s="15"/>
-      <c r="M80" s="15"/>
-      <c r="N80" s="15"/>
-      <c r="O80" s="15"/>
-      <c r="P80" s="15"/>
-      <c r="Q80" s="15"/>
+      <c r="J80" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="K80" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L80" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M80" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N80" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O80" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="P80" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q80" s="15" t="s">
+        <v>36</v>
+      </c>
       <c r="R80" s="15"/>
       <c r="S80" s="16" t="str">
         <f aca="false">IF(AND(G80&lt;&gt;"",COUNT(J80:N80)=5,OR(ISNUMBER(O80),O80="N/A"),P80&lt;&gt;"",Q80&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -24059,18 +24411,34 @@
       <c r="I81" s="14" t="s">
         <v>374</v>
       </c>
-      <c r="J81" s="15"/>
-      <c r="K81" s="15"/>
-      <c r="L81" s="15"/>
-      <c r="M81" s="15"/>
-      <c r="N81" s="15"/>
-      <c r="O81" s="15"/>
-      <c r="P81" s="15"/>
-      <c r="Q81" s="15"/>
+      <c r="J81" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="K81" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L81" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M81" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N81" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O81" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="P81" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q81" s="15" t="s">
+        <v>36</v>
+      </c>
       <c r="R81" s="15"/>
       <c r="S81" s="16" t="str">
         <f aca="false">IF(AND(G81&lt;&gt;"",COUNT(J81:N81)=5,OR(ISNUMBER(O81),O81="N/A"),P81&lt;&gt;"",Q81&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
[HUMAN-VALIDATION]: Increased number of validated test cases.
</commit_message>
<xml_diff>
--- a/thesis_evidence/validazione_umana/02_VALUTAZIONE_UMANA.xlsx
+++ b/thesis_evidence/validazione_umana/02_VALUTAZIONE_UMANA.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3025" uniqueCount="1071">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3088" uniqueCount="1071">
   <si>
     <t xml:space="preserve">Valutazione delle 250 risposte del test</t>
   </si>
@@ -20207,7 +20207,7 @@
       </c>
       <c r="B7" s="9" t="n">
         <f aca="false">COUNTIF(S9:S258,"OK")</f>
-        <v>73</v>
+        <v>102</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -24469,18 +24469,34 @@
       <c r="I82" s="14" t="s">
         <v>378</v>
       </c>
-      <c r="J82" s="15"/>
-      <c r="K82" s="15"/>
-      <c r="L82" s="15"/>
-      <c r="M82" s="15"/>
-      <c r="N82" s="15"/>
-      <c r="O82" s="15"/>
-      <c r="P82" s="15"/>
-      <c r="Q82" s="15"/>
+      <c r="J82" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="K82" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L82" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M82" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N82" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O82" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="P82" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q82" s="15" t="s">
+        <v>36</v>
+      </c>
       <c r="R82" s="15"/>
       <c r="S82" s="16" t="str">
         <f aca="false">IF(AND(G82&lt;&gt;"",COUNT(J82:N82)=5,OR(ISNUMBER(O82),O82="N/A"),P82&lt;&gt;"",Q82&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -24511,18 +24527,34 @@
       <c r="I83" s="14" t="s">
         <v>382</v>
       </c>
-      <c r="J83" s="15"/>
-      <c r="K83" s="15"/>
-      <c r="L83" s="15"/>
-      <c r="M83" s="15"/>
-      <c r="N83" s="15"/>
-      <c r="O83" s="15"/>
-      <c r="P83" s="15"/>
-      <c r="Q83" s="15"/>
+      <c r="J83" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="K83" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L83" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M83" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N83" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O83" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="P83" s="15" t="s">
+        <v>95</v>
+      </c>
+      <c r="Q83" s="15" t="s">
+        <v>75</v>
+      </c>
       <c r="R83" s="15"/>
       <c r="S83" s="16" t="str">
         <f aca="false">IF(AND(G83&lt;&gt;"",COUNT(J83:N83)=5,OR(ISNUMBER(O83),O83="N/A"),P83&lt;&gt;"",Q83&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -24553,18 +24585,34 @@
       <c r="I84" s="14" t="s">
         <v>386</v>
       </c>
-      <c r="J84" s="15"/>
-      <c r="K84" s="15"/>
-      <c r="L84" s="15"/>
-      <c r="M84" s="15"/>
-      <c r="N84" s="15"/>
-      <c r="O84" s="15"/>
-      <c r="P84" s="15"/>
-      <c r="Q84" s="15"/>
+      <c r="J84" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="K84" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L84" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M84" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N84" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O84" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="P84" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q84" s="15" t="s">
+        <v>36</v>
+      </c>
       <c r="R84" s="15"/>
       <c r="S84" s="16" t="str">
         <f aca="false">IF(AND(G84&lt;&gt;"",COUNT(J84:N84)=5,OR(ISNUMBER(O84),O84="N/A"),P84&lt;&gt;"",Q84&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -24595,18 +24643,34 @@
       <c r="I85" s="14" t="s">
         <v>390</v>
       </c>
-      <c r="J85" s="15"/>
-      <c r="K85" s="15"/>
-      <c r="L85" s="15"/>
-      <c r="M85" s="15"/>
-      <c r="N85" s="15"/>
-      <c r="O85" s="15"/>
-      <c r="P85" s="15"/>
-      <c r="Q85" s="15"/>
+      <c r="J85" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="K85" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L85" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M85" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N85" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O85" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="P85" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q85" s="15" t="s">
+        <v>36</v>
+      </c>
       <c r="R85" s="15"/>
       <c r="S85" s="16" t="str">
         <f aca="false">IF(AND(G85&lt;&gt;"",COUNT(J85:N85)=5,OR(ISNUMBER(O85),O85="N/A"),P85&lt;&gt;"",Q85&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -24637,18 +24701,34 @@
       <c r="I86" s="14" t="s">
         <v>396</v>
       </c>
-      <c r="J86" s="15"/>
-      <c r="K86" s="15"/>
-      <c r="L86" s="15"/>
-      <c r="M86" s="15"/>
-      <c r="N86" s="15"/>
-      <c r="O86" s="15"/>
-      <c r="P86" s="15"/>
-      <c r="Q86" s="15"/>
+      <c r="J86" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="K86" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L86" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M86" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N86" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O86" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="P86" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q86" s="15" t="s">
+        <v>36</v>
+      </c>
       <c r="R86" s="15"/>
       <c r="S86" s="16" t="str">
         <f aca="false">IF(AND(G86&lt;&gt;"",COUNT(J86:N86)=5,OR(ISNUMBER(O86),O86="N/A"),P86&lt;&gt;"",Q86&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -24679,18 +24759,34 @@
       <c r="I87" s="14" t="s">
         <v>400</v>
       </c>
-      <c r="J87" s="15"/>
-      <c r="K87" s="15"/>
-      <c r="L87" s="15"/>
-      <c r="M87" s="15"/>
-      <c r="N87" s="15"/>
-      <c r="O87" s="15"/>
-      <c r="P87" s="15"/>
-      <c r="Q87" s="15"/>
+      <c r="J87" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="K87" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L87" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M87" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N87" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O87" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="P87" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q87" s="15" t="s">
+        <v>36</v>
+      </c>
       <c r="R87" s="15"/>
       <c r="S87" s="16" t="str">
         <f aca="false">IF(AND(G87&lt;&gt;"",COUNT(J87:N87)=5,OR(ISNUMBER(O87),O87="N/A"),P87&lt;&gt;"",Q87&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -24717,18 +24813,34 @@
       </c>
       <c r="H88" s="14"/>
       <c r="I88" s="14"/>
-      <c r="J88" s="15"/>
-      <c r="K88" s="15"/>
-      <c r="L88" s="15"/>
-      <c r="M88" s="15"/>
-      <c r="N88" s="15"/>
-      <c r="O88" s="15"/>
-      <c r="P88" s="15"/>
-      <c r="Q88" s="15"/>
+      <c r="J88" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="K88" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L88" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M88" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N88" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O88" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="P88" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q88" s="15" t="s">
+        <v>36</v>
+      </c>
       <c r="R88" s="15"/>
       <c r="S88" s="16" t="str">
         <f aca="false">IF(AND(G88&lt;&gt;"",COUNT(J88:N88)=5,OR(ISNUMBER(O88),O88="N/A"),P88&lt;&gt;"",Q88&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -24759,18 +24871,34 @@
       <c r="I89" s="14" t="s">
         <v>406</v>
       </c>
-      <c r="J89" s="15"/>
-      <c r="K89" s="15"/>
-      <c r="L89" s="15"/>
-      <c r="M89" s="15"/>
-      <c r="N89" s="15"/>
-      <c r="O89" s="15"/>
-      <c r="P89" s="15"/>
-      <c r="Q89" s="15"/>
+      <c r="J89" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="K89" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L89" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M89" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N89" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O89" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="P89" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q89" s="15" t="s">
+        <v>36</v>
+      </c>
       <c r="R89" s="15"/>
       <c r="S89" s="16" t="str">
         <f aca="false">IF(AND(G89&lt;&gt;"",COUNT(J89:N89)=5,OR(ISNUMBER(O89),O89="N/A"),P89&lt;&gt;"",Q89&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -24797,18 +24925,34 @@
       </c>
       <c r="H90" s="14"/>
       <c r="I90" s="14"/>
-      <c r="J90" s="15"/>
-      <c r="K90" s="15"/>
-      <c r="L90" s="15"/>
-      <c r="M90" s="15"/>
-      <c r="N90" s="15"/>
-      <c r="O90" s="15"/>
-      <c r="P90" s="15"/>
-      <c r="Q90" s="15"/>
+      <c r="J90" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="K90" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L90" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M90" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N90" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O90" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="P90" s="15" t="s">
+        <v>74</v>
+      </c>
+      <c r="Q90" s="15" t="s">
+        <v>104</v>
+      </c>
       <c r="R90" s="15"/>
       <c r="S90" s="16" t="str">
         <f aca="false">IF(AND(G90&lt;&gt;"",COUNT(J90:N90)=5,OR(ISNUMBER(O90),O90="N/A"),P90&lt;&gt;"",Q90&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -24835,18 +24979,34 @@
       </c>
       <c r="H91" s="14"/>
       <c r="I91" s="14"/>
-      <c r="J91" s="15"/>
-      <c r="K91" s="15"/>
-      <c r="L91" s="15"/>
-      <c r="M91" s="15"/>
-      <c r="N91" s="15"/>
-      <c r="O91" s="15"/>
-      <c r="P91" s="15"/>
-      <c r="Q91" s="15"/>
+      <c r="J91" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="K91" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L91" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M91" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N91" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O91" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="P91" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q91" s="15" t="s">
+        <v>36</v>
+      </c>
       <c r="R91" s="15"/>
       <c r="S91" s="16" t="str">
         <f aca="false">IF(AND(G91&lt;&gt;"",COUNT(J91:N91)=5,OR(ISNUMBER(O91),O91="N/A"),P91&lt;&gt;"",Q91&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -24877,18 +25037,34 @@
       <c r="I92" s="14" t="s">
         <v>416</v>
       </c>
-      <c r="J92" s="15"/>
-      <c r="K92" s="15"/>
-      <c r="L92" s="15"/>
-      <c r="M92" s="15"/>
-      <c r="N92" s="15"/>
-      <c r="O92" s="15"/>
-      <c r="P92" s="15"/>
-      <c r="Q92" s="15"/>
+      <c r="J92" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="K92" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L92" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M92" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N92" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O92" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="P92" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q92" s="15" t="s">
+        <v>36</v>
+      </c>
       <c r="R92" s="15"/>
       <c r="S92" s="16" t="str">
         <f aca="false">IF(AND(G92&lt;&gt;"",COUNT(J92:N92)=5,OR(ISNUMBER(O92),O92="N/A"),P92&lt;&gt;"",Q92&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -24919,18 +25095,34 @@
       <c r="I93" s="14" t="s">
         <v>420</v>
       </c>
-      <c r="J93" s="15"/>
-      <c r="K93" s="15"/>
-      <c r="L93" s="15"/>
-      <c r="M93" s="15"/>
-      <c r="N93" s="15"/>
-      <c r="O93" s="15"/>
-      <c r="P93" s="15"/>
-      <c r="Q93" s="15"/>
+      <c r="J93" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="K93" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L93" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M93" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N93" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O93" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="P93" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q93" s="15" t="s">
+        <v>75</v>
+      </c>
       <c r="R93" s="15"/>
       <c r="S93" s="16" t="str">
         <f aca="false">IF(AND(G93&lt;&gt;"",COUNT(J93:N93)=5,OR(ISNUMBER(O93),O93="N/A"),P93&lt;&gt;"",Q93&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -24957,18 +25149,34 @@
       </c>
       <c r="H94" s="14"/>
       <c r="I94" s="14"/>
-      <c r="J94" s="15"/>
-      <c r="K94" s="15"/>
-      <c r="L94" s="15"/>
-      <c r="M94" s="15"/>
-      <c r="N94" s="15"/>
-      <c r="O94" s="15"/>
-      <c r="P94" s="15"/>
-      <c r="Q94" s="15"/>
+      <c r="J94" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="K94" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L94" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M94" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N94" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O94" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="P94" s="15" t="s">
+        <v>95</v>
+      </c>
+      <c r="Q94" s="15" t="s">
+        <v>36</v>
+      </c>
       <c r="R94" s="15"/>
       <c r="S94" s="16" t="str">
         <f aca="false">IF(AND(G94&lt;&gt;"",COUNT(J94:N94)=5,OR(ISNUMBER(O94),O94="N/A"),P94&lt;&gt;"",Q94&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -24999,18 +25207,34 @@
       <c r="I95" s="14" t="s">
         <v>426</v>
       </c>
-      <c r="J95" s="15"/>
-      <c r="K95" s="15"/>
-      <c r="L95" s="15"/>
-      <c r="M95" s="15"/>
-      <c r="N95" s="15"/>
-      <c r="O95" s="15"/>
-      <c r="P95" s="15"/>
-      <c r="Q95" s="15"/>
+      <c r="J95" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="K95" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L95" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M95" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N95" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O95" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="P95" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q95" s="15" t="s">
+        <v>36</v>
+      </c>
       <c r="R95" s="15"/>
       <c r="S95" s="16" t="str">
         <f aca="false">IF(AND(G95&lt;&gt;"",COUNT(J95:N95)=5,OR(ISNUMBER(O95),O95="N/A"),P95&lt;&gt;"",Q95&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -25041,18 +25265,34 @@
       <c r="I96" s="14" t="s">
         <v>430</v>
       </c>
-      <c r="J96" s="15"/>
-      <c r="K96" s="15"/>
-      <c r="L96" s="15"/>
-      <c r="M96" s="15"/>
-      <c r="N96" s="15"/>
-      <c r="O96" s="15"/>
-      <c r="P96" s="15"/>
-      <c r="Q96" s="15"/>
+      <c r="J96" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="K96" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L96" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M96" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N96" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O96" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="P96" s="15" t="s">
+        <v>95</v>
+      </c>
+      <c r="Q96" s="15" t="s">
+        <v>75</v>
+      </c>
       <c r="R96" s="15"/>
       <c r="S96" s="16" t="str">
         <f aca="false">IF(AND(G96&lt;&gt;"",COUNT(J96:N96)=5,OR(ISNUMBER(O96),O96="N/A"),P96&lt;&gt;"",Q96&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -25083,18 +25323,34 @@
       <c r="I97" s="14" t="s">
         <v>434</v>
       </c>
-      <c r="J97" s="15"/>
-      <c r="K97" s="15"/>
-      <c r="L97" s="15"/>
-      <c r="M97" s="15"/>
-      <c r="N97" s="15"/>
-      <c r="O97" s="15"/>
-      <c r="P97" s="15"/>
-      <c r="Q97" s="15"/>
+      <c r="J97" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="K97" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L97" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M97" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N97" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O97" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="P97" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q97" s="15" t="s">
+        <v>36</v>
+      </c>
       <c r="R97" s="15"/>
       <c r="S97" s="16" t="str">
         <f aca="false">IF(AND(G97&lt;&gt;"",COUNT(J97:N97)=5,OR(ISNUMBER(O97),O97="N/A"),P97&lt;&gt;"",Q97&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -25125,18 +25381,34 @@
       <c r="I98" s="14" t="s">
         <v>439</v>
       </c>
-      <c r="J98" s="15"/>
-      <c r="K98" s="15"/>
-      <c r="L98" s="15"/>
-      <c r="M98" s="15"/>
-      <c r="N98" s="15"/>
-      <c r="O98" s="15"/>
-      <c r="P98" s="15"/>
-      <c r="Q98" s="15"/>
+      <c r="J98" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="K98" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L98" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M98" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N98" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O98" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="P98" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q98" s="15" t="s">
+        <v>36</v>
+      </c>
       <c r="R98" s="15"/>
       <c r="S98" s="16" t="str">
         <f aca="false">IF(AND(G98&lt;&gt;"",COUNT(J98:N98)=5,OR(ISNUMBER(O98),O98="N/A"),P98&lt;&gt;"",Q98&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -25167,18 +25439,34 @@
       <c r="I99" s="14" t="s">
         <v>443</v>
       </c>
-      <c r="J99" s="15"/>
-      <c r="K99" s="15"/>
-      <c r="L99" s="15"/>
-      <c r="M99" s="15"/>
-      <c r="N99" s="15"/>
-      <c r="O99" s="15"/>
-      <c r="P99" s="15"/>
-      <c r="Q99" s="15"/>
+      <c r="J99" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="K99" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L99" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M99" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N99" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O99" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="P99" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q99" s="15" t="s">
+        <v>36</v>
+      </c>
       <c r="R99" s="15"/>
       <c r="S99" s="16" t="str">
         <f aca="false">IF(AND(G99&lt;&gt;"",COUNT(J99:N99)=5,OR(ISNUMBER(O99),O99="N/A"),P99&lt;&gt;"",Q99&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="100" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -25209,18 +25497,34 @@
       <c r="I100" s="14" t="s">
         <v>447</v>
       </c>
-      <c r="J100" s="15"/>
-      <c r="K100" s="15"/>
-      <c r="L100" s="15"/>
-      <c r="M100" s="15"/>
-      <c r="N100" s="15"/>
-      <c r="O100" s="15"/>
-      <c r="P100" s="15"/>
-      <c r="Q100" s="15"/>
+      <c r="J100" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="K100" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L100" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M100" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N100" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O100" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="P100" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q100" s="15" t="s">
+        <v>36</v>
+      </c>
       <c r="R100" s="15"/>
       <c r="S100" s="16" t="str">
         <f aca="false">IF(AND(G100&lt;&gt;"",COUNT(J100:N100)=5,OR(ISNUMBER(O100),O100="N/A"),P100&lt;&gt;"",Q100&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -25251,18 +25555,34 @@
       <c r="I101" s="14" t="s">
         <v>451</v>
       </c>
-      <c r="J101" s="15"/>
-      <c r="K101" s="15"/>
-      <c r="L101" s="15"/>
-      <c r="M101" s="15"/>
-      <c r="N101" s="15"/>
-      <c r="O101" s="15"/>
-      <c r="P101" s="15"/>
-      <c r="Q101" s="15"/>
+      <c r="J101" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="K101" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L101" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M101" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N101" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O101" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="P101" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q101" s="15" t="s">
+        <v>36</v>
+      </c>
       <c r="R101" s="15"/>
       <c r="S101" s="16" t="str">
         <f aca="false">IF(AND(G101&lt;&gt;"",COUNT(J101:N101)=5,OR(ISNUMBER(O101),O101="N/A"),P101&lt;&gt;"",Q101&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -25289,18 +25609,34 @@
       </c>
       <c r="H102" s="14"/>
       <c r="I102" s="14"/>
-      <c r="J102" s="15"/>
-      <c r="K102" s="15"/>
-      <c r="L102" s="15"/>
-      <c r="M102" s="15"/>
-      <c r="N102" s="15"/>
-      <c r="O102" s="15"/>
-      <c r="P102" s="15"/>
-      <c r="Q102" s="15"/>
+      <c r="J102" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="K102" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L102" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M102" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N102" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O102" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="P102" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q102" s="15" t="s">
+        <v>125</v>
+      </c>
       <c r="R102" s="15"/>
       <c r="S102" s="16" t="str">
         <f aca="false">IF(AND(G102&lt;&gt;"",COUNT(J102:N102)=5,OR(ISNUMBER(O102),O102="N/A"),P102&lt;&gt;"",Q102&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="103" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -25331,18 +25667,34 @@
       <c r="I103" s="14" t="s">
         <v>457</v>
       </c>
-      <c r="J103" s="15"/>
-      <c r="K103" s="15"/>
-      <c r="L103" s="15"/>
-      <c r="M103" s="15"/>
-      <c r="N103" s="15"/>
-      <c r="O103" s="15"/>
-      <c r="P103" s="15"/>
-      <c r="Q103" s="15"/>
+      <c r="J103" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="K103" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="L103" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M103" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N103" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O103" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="P103" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q103" s="15" t="s">
+        <v>75</v>
+      </c>
       <c r="R103" s="15"/>
       <c r="S103" s="16" t="str">
         <f aca="false">IF(AND(G103&lt;&gt;"",COUNT(J103:N103)=5,OR(ISNUMBER(O103),O103="N/A"),P103&lt;&gt;"",Q103&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -25373,18 +25725,34 @@
       <c r="I104" s="14" t="s">
         <v>461</v>
       </c>
-      <c r="J104" s="15"/>
-      <c r="K104" s="15"/>
-      <c r="L104" s="15"/>
-      <c r="M104" s="15"/>
-      <c r="N104" s="15"/>
-      <c r="O104" s="15"/>
-      <c r="P104" s="15"/>
-      <c r="Q104" s="15"/>
+      <c r="J104" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="K104" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L104" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M104" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N104" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O104" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="P104" s="15" t="s">
+        <v>95</v>
+      </c>
+      <c r="Q104" s="15" t="s">
+        <v>75</v>
+      </c>
       <c r="R104" s="15"/>
       <c r="S104" s="16" t="str">
         <f aca="false">IF(AND(G104&lt;&gt;"",COUNT(J104:N104)=5,OR(ISNUMBER(O104),O104="N/A"),P104&lt;&gt;"",Q104&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="105" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -25415,18 +25783,34 @@
       <c r="I105" s="14" t="s">
         <v>466</v>
       </c>
-      <c r="J105" s="15"/>
-      <c r="K105" s="15"/>
-      <c r="L105" s="15"/>
-      <c r="M105" s="15"/>
-      <c r="N105" s="15"/>
-      <c r="O105" s="15"/>
-      <c r="P105" s="15"/>
-      <c r="Q105" s="15"/>
+      <c r="J105" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="K105" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L105" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M105" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N105" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O105" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="P105" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q105" s="15" t="s">
+        <v>36</v>
+      </c>
       <c r="R105" s="15"/>
       <c r="S105" s="16" t="str">
         <f aca="false">IF(AND(G105&lt;&gt;"",COUNT(J105:N105)=5,OR(ISNUMBER(O105),O105="N/A"),P105&lt;&gt;"",Q105&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="106" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -25457,18 +25841,34 @@
       <c r="I106" s="14" t="s">
         <v>471</v>
       </c>
-      <c r="J106" s="15"/>
-      <c r="K106" s="15"/>
-      <c r="L106" s="15"/>
-      <c r="M106" s="15"/>
-      <c r="N106" s="15"/>
-      <c r="O106" s="15"/>
-      <c r="P106" s="15"/>
-      <c r="Q106" s="15"/>
+      <c r="J106" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="K106" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L106" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M106" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N106" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O106" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="P106" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q106" s="15" t="s">
+        <v>36</v>
+      </c>
       <c r="R106" s="15"/>
       <c r="S106" s="16" t="str">
         <f aca="false">IF(AND(G106&lt;&gt;"",COUNT(J106:N106)=5,OR(ISNUMBER(O106),O106="N/A"),P106&lt;&gt;"",Q106&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="107" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -25499,18 +25899,34 @@
       <c r="I107" s="14" t="s">
         <v>475</v>
       </c>
-      <c r="J107" s="15"/>
-      <c r="K107" s="15"/>
-      <c r="L107" s="15"/>
-      <c r="M107" s="15"/>
-      <c r="N107" s="15"/>
-      <c r="O107" s="15"/>
-      <c r="P107" s="15"/>
-      <c r="Q107" s="15"/>
+      <c r="J107" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="K107" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L107" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M107" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N107" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O107" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="P107" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q107" s="15" t="s">
+        <v>36</v>
+      </c>
       <c r="R107" s="15"/>
       <c r="S107" s="16" t="str">
         <f aca="false">IF(AND(G107&lt;&gt;"",COUNT(J107:N107)=5,OR(ISNUMBER(O107),O107="N/A"),P107&lt;&gt;"",Q107&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="108" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -25541,18 +25957,34 @@
       <c r="I108" s="14" t="s">
         <v>479</v>
       </c>
-      <c r="J108" s="15"/>
-      <c r="K108" s="15"/>
-      <c r="L108" s="15"/>
-      <c r="M108" s="15"/>
-      <c r="N108" s="15"/>
-      <c r="O108" s="15"/>
-      <c r="P108" s="15"/>
-      <c r="Q108" s="15"/>
+      <c r="J108" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="K108" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L108" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M108" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N108" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O108" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="P108" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q108" s="15" t="s">
+        <v>36</v>
+      </c>
       <c r="R108" s="15"/>
       <c r="S108" s="16" t="str">
         <f aca="false">IF(AND(G108&lt;&gt;"",COUNT(J108:N108)=5,OR(ISNUMBER(O108),O108="N/A"),P108&lt;&gt;"",Q108&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="109" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -25583,18 +26015,34 @@
       <c r="I109" s="14" t="s">
         <v>483</v>
       </c>
-      <c r="J109" s="15"/>
-      <c r="K109" s="15"/>
-      <c r="L109" s="15"/>
-      <c r="M109" s="15"/>
-      <c r="N109" s="15"/>
-      <c r="O109" s="15"/>
-      <c r="P109" s="15"/>
-      <c r="Q109" s="15"/>
+      <c r="J109" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="K109" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="L109" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M109" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N109" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O109" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="P109" s="15" t="s">
+        <v>95</v>
+      </c>
+      <c r="Q109" s="15" t="s">
+        <v>75</v>
+      </c>
       <c r="R109" s="15"/>
       <c r="S109" s="16" t="str">
         <f aca="false">IF(AND(G109&lt;&gt;"",COUNT(J109:N109)=5,OR(ISNUMBER(O109),O109="N/A"),P109&lt;&gt;"",Q109&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="110" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -25625,18 +26073,34 @@
       <c r="I110" s="14" t="s">
         <v>487</v>
       </c>
-      <c r="J110" s="15"/>
-      <c r="K110" s="15"/>
-      <c r="L110" s="15"/>
-      <c r="M110" s="15"/>
-      <c r="N110" s="15"/>
-      <c r="O110" s="15"/>
-      <c r="P110" s="15"/>
-      <c r="Q110" s="15"/>
+      <c r="J110" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="K110" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L110" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M110" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N110" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O110" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="P110" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q110" s="15" t="s">
+        <v>36</v>
+      </c>
       <c r="R110" s="15"/>
       <c r="S110" s="16" t="str">
         <f aca="false">IF(AND(G110&lt;&gt;"",COUNT(J110:N110)=5,OR(ISNUMBER(O110),O110="N/A"),P110&lt;&gt;"",Q110&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="111" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -31752,36 +32216,68 @@
       <formula>NOT(ISERROR(SEARCH("DA COMPLETARE",S9)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="8">
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J9:J258" type="list">
+  <dataValidations count="16">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J9:J81 J111:J258" type="list">
       <formula1>"0,1,2,3"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="K9:K258" type="list">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="K9:K81 K111:K258" type="list">
       <formula1>"0,1,2,3"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="L9:L258" type="list">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="L9:L81 L111:L258" type="list">
       <formula1>"0,1,2,3"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="M9:M258" type="list">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="M9:M81 M111:M258" type="list">
       <formula1>"0,1,2,3"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="N9:N258" type="list">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="N9:N81 N111:N258" type="list">
       <formula1>"0,1,2,3"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="O9:O258" type="list">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="O9:O81 O111:O258" type="list">
       <formula1>"0,1,2,3,N/A"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="P9:P258" type="list">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="P9:P81 P111:P258" type="list">
       <formula1>"CORRETTA,PARZIALMENTE_CORRETTA,ERRATA,NON_INDICATA"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="Q9:Q258" type="list">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="Q9:Q81 Q111:Q258" type="list">
+      <formula1>"NESSUNO,SOURCE_NOT_RETRIEVED,SOURCE_OUTSIDE_TOP_K,SOURCE_IN_PROMPT_IGNORED,TELEMETRY_MISINTERPRETED,WRONG_ROOT_CAUSE,INVALID_CITATION,UNSUPPORTED_CLAIM,INCOMPLETE_RESPONSE,UNSAFE_ACTION"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J82:J110" type="list">
+      <formula1>"0,1,2,3"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="K82:K110" type="list">
+      <formula1>"0,1,2,3"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="L82:L110" type="list">
+      <formula1>"0,1,2,3"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="M82:M110" type="list">
+      <formula1>"0,1,2,3"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="N82:N110" type="list">
+      <formula1>"0,1,2,3"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="O82:O110" type="list">
+      <formula1>"0,1,2,3,N/A"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="P82:P110" type="list">
+      <formula1>"CORRETTA,PARZIALMENTE_CORRETTA,ERRATA,NON_INDICATA"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="Q82:Q110" type="list">
       <formula1>"NESSUNO,SOURCE_NOT_RETRIEVED,SOURCE_OUTSIDE_TOP_K,SOURCE_IN_PROMPT_IGNORED,TELEMETRY_MISINTERPRETED,WRONG_ROOT_CAUSE,INVALID_CITATION,UNSUPPORTED_CLAIM,INCOMPLETE_RESPONSE,UNSAFE_ACTION"</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>

<commit_message>
[HUMAN-VALIDATION]: Increased test cases validated.
</commit_message>
<xml_diff>
--- a/thesis_evidence/validazione_umana/02_VALUTAZIONE_UMANA.xlsx
+++ b/thesis_evidence/validazione_umana/02_VALUTAZIONE_UMANA.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3088" uniqueCount="1071">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3163" uniqueCount="1071">
   <si>
     <t xml:space="preserve">Valutazione delle 250 risposte del test</t>
   </si>
@@ -20207,7 +20207,7 @@
       </c>
       <c r="B7" s="9" t="n">
         <f aca="false">COUNTIF(S9:S258,"OK")</f>
-        <v>102</v>
+        <v>136</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -26127,18 +26127,34 @@
       </c>
       <c r="H111" s="14"/>
       <c r="I111" s="14"/>
-      <c r="J111" s="15"/>
-      <c r="K111" s="15"/>
-      <c r="L111" s="15"/>
-      <c r="M111" s="15"/>
-      <c r="N111" s="15"/>
-      <c r="O111" s="15"/>
-      <c r="P111" s="15"/>
-      <c r="Q111" s="15"/>
+      <c r="J111" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="K111" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="L111" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M111" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N111" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O111" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="P111" s="15" t="s">
+        <v>95</v>
+      </c>
+      <c r="Q111" s="15" t="s">
+        <v>125</v>
+      </c>
       <c r="R111" s="15"/>
       <c r="S111" s="16" t="str">
         <f aca="false">IF(AND(G111&lt;&gt;"",COUNT(J111:N111)=5,OR(ISNUMBER(O111),O111="N/A"),P111&lt;&gt;"",Q111&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="112" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -26169,18 +26185,34 @@
       <c r="I112" s="14" t="s">
         <v>493</v>
       </c>
-      <c r="J112" s="15"/>
-      <c r="K112" s="15"/>
-      <c r="L112" s="15"/>
-      <c r="M112" s="15"/>
-      <c r="N112" s="15"/>
-      <c r="O112" s="15"/>
-      <c r="P112" s="15"/>
-      <c r="Q112" s="15"/>
+      <c r="J112" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="K112" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L112" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M112" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N112" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O112" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="P112" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q112" s="15" t="s">
+        <v>36</v>
+      </c>
       <c r="R112" s="15"/>
       <c r="S112" s="16" t="str">
         <f aca="false">IF(AND(G112&lt;&gt;"",COUNT(J112:N112)=5,OR(ISNUMBER(O112),O112="N/A"),P112&lt;&gt;"",Q112&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="113" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -26211,18 +26243,34 @@
       <c r="I113" s="14" t="s">
         <v>497</v>
       </c>
-      <c r="J113" s="15"/>
-      <c r="K113" s="15"/>
-      <c r="L113" s="15"/>
-      <c r="M113" s="15"/>
-      <c r="N113" s="15"/>
-      <c r="O113" s="15"/>
-      <c r="P113" s="15"/>
-      <c r="Q113" s="15"/>
+      <c r="J113" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="K113" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L113" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M113" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N113" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O113" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="P113" s="15" t="s">
+        <v>95</v>
+      </c>
+      <c r="Q113" s="15" t="s">
+        <v>75</v>
+      </c>
       <c r="R113" s="15"/>
       <c r="S113" s="16" t="str">
         <f aca="false">IF(AND(G113&lt;&gt;"",COUNT(J113:N113)=5,OR(ISNUMBER(O113),O113="N/A"),P113&lt;&gt;"",Q113&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="114" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -26253,18 +26301,34 @@
       <c r="I114" s="14" t="s">
         <v>501</v>
       </c>
-      <c r="J114" s="15"/>
-      <c r="K114" s="15"/>
-      <c r="L114" s="15"/>
-      <c r="M114" s="15"/>
-      <c r="N114" s="15"/>
-      <c r="O114" s="15"/>
-      <c r="P114" s="15"/>
-      <c r="Q114" s="15"/>
+      <c r="J114" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="K114" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L114" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M114" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N114" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O114" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="P114" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q114" s="15" t="s">
+        <v>36</v>
+      </c>
       <c r="R114" s="15"/>
       <c r="S114" s="16" t="str">
         <f aca="false">IF(AND(G114&lt;&gt;"",COUNT(J114:N114)=5,OR(ISNUMBER(O114),O114="N/A"),P114&lt;&gt;"",Q114&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="115" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -26295,18 +26359,34 @@
       <c r="I115" s="14" t="s">
         <v>507</v>
       </c>
-      <c r="J115" s="15"/>
-      <c r="K115" s="15"/>
-      <c r="L115" s="15"/>
-      <c r="M115" s="15"/>
-      <c r="N115" s="15"/>
-      <c r="O115" s="15"/>
-      <c r="P115" s="15"/>
-      <c r="Q115" s="15"/>
+      <c r="J115" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="K115" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L115" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M115" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N115" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O115" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="P115" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q115" s="15" t="s">
+        <v>36</v>
+      </c>
       <c r="R115" s="15"/>
       <c r="S115" s="16" t="str">
         <f aca="false">IF(AND(G115&lt;&gt;"",COUNT(J115:N115)=5,OR(ISNUMBER(O115),O115="N/A"),P115&lt;&gt;"",Q115&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="116" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -26333,18 +26413,34 @@
       </c>
       <c r="H116" s="14"/>
       <c r="I116" s="14"/>
-      <c r="J116" s="15"/>
-      <c r="K116" s="15"/>
-      <c r="L116" s="15"/>
-      <c r="M116" s="15"/>
-      <c r="N116" s="15"/>
-      <c r="O116" s="15"/>
-      <c r="P116" s="15"/>
-      <c r="Q116" s="15"/>
+      <c r="J116" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="K116" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L116" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M116" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N116" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O116" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="P116" s="15" t="s">
+        <v>95</v>
+      </c>
+      <c r="Q116" s="15" t="s">
+        <v>36</v>
+      </c>
       <c r="R116" s="15"/>
       <c r="S116" s="16" t="str">
         <f aca="false">IF(AND(G116&lt;&gt;"",COUNT(J116:N116)=5,OR(ISNUMBER(O116),O116="N/A"),P116&lt;&gt;"",Q116&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="117" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -26375,18 +26471,34 @@
       <c r="I117" s="14" t="s">
         <v>514</v>
       </c>
-      <c r="J117" s="15"/>
-      <c r="K117" s="15"/>
-      <c r="L117" s="15"/>
-      <c r="M117" s="15"/>
-      <c r="N117" s="15"/>
-      <c r="O117" s="15"/>
-      <c r="P117" s="15"/>
-      <c r="Q117" s="15"/>
+      <c r="J117" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="K117" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L117" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M117" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N117" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O117" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="P117" s="15" t="s">
+        <v>116</v>
+      </c>
+      <c r="Q117" s="15" t="s">
+        <v>117</v>
+      </c>
       <c r="R117" s="15"/>
       <c r="S117" s="16" t="str">
         <f aca="false">IF(AND(G117&lt;&gt;"",COUNT(J117:N117)=5,OR(ISNUMBER(O117),O117="N/A"),P117&lt;&gt;"",Q117&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="118" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -26417,18 +26529,34 @@
       <c r="I118" s="14" t="s">
         <v>518</v>
       </c>
-      <c r="J118" s="15"/>
-      <c r="K118" s="15"/>
-      <c r="L118" s="15"/>
-      <c r="M118" s="15"/>
-      <c r="N118" s="15"/>
-      <c r="O118" s="15"/>
-      <c r="P118" s="15"/>
-      <c r="Q118" s="15"/>
+      <c r="J118" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="K118" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="L118" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M118" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N118" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="O118" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="P118" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q118" s="15" t="s">
+        <v>36</v>
+      </c>
       <c r="R118" s="15"/>
       <c r="S118" s="16" t="str">
         <f aca="false">IF(AND(G118&lt;&gt;"",COUNT(J118:N118)=5,OR(ISNUMBER(O118),O118="N/A"),P118&lt;&gt;"",Q118&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="119" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -26459,18 +26587,34 @@
       <c r="I119" s="14" t="s">
         <v>522</v>
       </c>
-      <c r="J119" s="15"/>
-      <c r="K119" s="15"/>
-      <c r="L119" s="15"/>
-      <c r="M119" s="15"/>
-      <c r="N119" s="15"/>
-      <c r="O119" s="15"/>
-      <c r="P119" s="15"/>
-      <c r="Q119" s="15"/>
+      <c r="J119" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="K119" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="L119" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M119" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N119" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O119" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="P119" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q119" s="15" t="s">
+        <v>75</v>
+      </c>
       <c r="R119" s="15"/>
       <c r="S119" s="16" t="str">
         <f aca="false">IF(AND(G119&lt;&gt;"",COUNT(J119:N119)=5,OR(ISNUMBER(O119),O119="N/A"),P119&lt;&gt;"",Q119&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="120" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -26501,18 +26645,34 @@
       <c r="I120" s="14" t="s">
         <v>526</v>
       </c>
-      <c r="J120" s="15"/>
-      <c r="K120" s="15"/>
-      <c r="L120" s="15"/>
-      <c r="M120" s="15"/>
-      <c r="N120" s="15"/>
-      <c r="O120" s="15"/>
-      <c r="P120" s="15"/>
-      <c r="Q120" s="15"/>
+      <c r="J120" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="K120" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L120" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M120" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N120" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O120" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="P120" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q120" s="15" t="s">
+        <v>36</v>
+      </c>
       <c r="R120" s="15"/>
       <c r="S120" s="16" t="str">
         <f aca="false">IF(AND(G120&lt;&gt;"",COUNT(J120:N120)=5,OR(ISNUMBER(O120),O120="N/A"),P120&lt;&gt;"",Q120&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="121" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -26543,18 +26703,34 @@
       <c r="I121" s="14" t="s">
         <v>530</v>
       </c>
-      <c r="J121" s="15"/>
-      <c r="K121" s="15"/>
-      <c r="L121" s="15"/>
-      <c r="M121" s="15"/>
-      <c r="N121" s="15"/>
-      <c r="O121" s="15"/>
-      <c r="P121" s="15"/>
-      <c r="Q121" s="15"/>
+      <c r="J121" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="K121" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L121" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M121" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N121" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O121" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="P121" s="15" t="s">
+        <v>95</v>
+      </c>
+      <c r="Q121" s="15" t="s">
+        <v>36</v>
+      </c>
       <c r="R121" s="15"/>
       <c r="S121" s="16" t="str">
         <f aca="false">IF(AND(G121&lt;&gt;"",COUNT(J121:N121)=5,OR(ISNUMBER(O121),O121="N/A"),P121&lt;&gt;"",Q121&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="122" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -26585,18 +26761,34 @@
       <c r="I122" s="14" t="s">
         <v>534</v>
       </c>
-      <c r="J122" s="15"/>
-      <c r="K122" s="15"/>
-      <c r="L122" s="15"/>
-      <c r="M122" s="15"/>
-      <c r="N122" s="15"/>
-      <c r="O122" s="15"/>
-      <c r="P122" s="15"/>
-      <c r="Q122" s="15"/>
+      <c r="J122" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="K122" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L122" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M122" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N122" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O122" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="P122" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q122" s="15" t="s">
+        <v>36</v>
+      </c>
       <c r="R122" s="15"/>
       <c r="S122" s="16" t="str">
         <f aca="false">IF(AND(G122&lt;&gt;"",COUNT(J122:N122)=5,OR(ISNUMBER(O122),O122="N/A"),P122&lt;&gt;"",Q122&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="123" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -26627,18 +26819,34 @@
       <c r="I123" s="14" t="s">
         <v>538</v>
       </c>
-      <c r="J123" s="15"/>
-      <c r="K123" s="15"/>
-      <c r="L123" s="15"/>
-      <c r="M123" s="15"/>
-      <c r="N123" s="15"/>
-      <c r="O123" s="15"/>
-      <c r="P123" s="15"/>
-      <c r="Q123" s="15"/>
+      <c r="J123" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="K123" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L123" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M123" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N123" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O123" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="P123" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q123" s="15" t="s">
+        <v>36</v>
+      </c>
       <c r="R123" s="15"/>
       <c r="S123" s="16" t="str">
         <f aca="false">IF(AND(G123&lt;&gt;"",COUNT(J123:N123)=5,OR(ISNUMBER(O123),O123="N/A"),P123&lt;&gt;"",Q123&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="124" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -26665,18 +26873,34 @@
       </c>
       <c r="H124" s="14"/>
       <c r="I124" s="14"/>
-      <c r="J124" s="15"/>
-      <c r="K124" s="15"/>
-      <c r="L124" s="15"/>
-      <c r="M124" s="15"/>
-      <c r="N124" s="15"/>
-      <c r="O124" s="15"/>
-      <c r="P124" s="15"/>
-      <c r="Q124" s="15"/>
+      <c r="J124" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="K124" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L124" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M124" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N124" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O124" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="P124" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q124" s="15" t="s">
+        <v>36</v>
+      </c>
       <c r="R124" s="15"/>
       <c r="S124" s="16" t="str">
         <f aca="false">IF(AND(G124&lt;&gt;"",COUNT(J124:N124)=5,OR(ISNUMBER(O124),O124="N/A"),P124&lt;&gt;"",Q124&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="125" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -26707,18 +26931,34 @@
       <c r="I125" s="14" t="s">
         <v>543</v>
       </c>
-      <c r="J125" s="15"/>
-      <c r="K125" s="15"/>
-      <c r="L125" s="15"/>
-      <c r="M125" s="15"/>
-      <c r="N125" s="15"/>
-      <c r="O125" s="15"/>
-      <c r="P125" s="15"/>
-      <c r="Q125" s="15"/>
+      <c r="J125" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="K125" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L125" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M125" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N125" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O125" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="P125" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q125" s="15" t="s">
+        <v>75</v>
+      </c>
       <c r="R125" s="15"/>
       <c r="S125" s="16" t="str">
         <f aca="false">IF(AND(G125&lt;&gt;"",COUNT(J125:N125)=5,OR(ISNUMBER(O125),O125="N/A"),P125&lt;&gt;"",Q125&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="126" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -26749,18 +26989,34 @@
       <c r="I126" s="14" t="s">
         <v>547</v>
       </c>
-      <c r="J126" s="15"/>
-      <c r="K126" s="15"/>
-      <c r="L126" s="15"/>
-      <c r="M126" s="15"/>
-      <c r="N126" s="15"/>
-      <c r="O126" s="15"/>
-      <c r="P126" s="15"/>
-      <c r="Q126" s="15"/>
+      <c r="J126" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="K126" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L126" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M126" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N126" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O126" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="P126" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q126" s="15" t="s">
+        <v>36</v>
+      </c>
       <c r="R126" s="15"/>
       <c r="S126" s="16" t="str">
         <f aca="false">IF(AND(G126&lt;&gt;"",COUNT(J126:N126)=5,OR(ISNUMBER(O126),O126="N/A"),P126&lt;&gt;"",Q126&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="127" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -26791,18 +27047,34 @@
       <c r="I127" s="14" t="s">
         <v>551</v>
       </c>
-      <c r="J127" s="15"/>
-      <c r="K127" s="15"/>
-      <c r="L127" s="15"/>
-      <c r="M127" s="15"/>
-      <c r="N127" s="15"/>
-      <c r="O127" s="15"/>
-      <c r="P127" s="15"/>
-      <c r="Q127" s="15"/>
+      <c r="J127" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="K127" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L127" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M127" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N127" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O127" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="P127" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q127" s="15" t="s">
+        <v>36</v>
+      </c>
       <c r="R127" s="15"/>
       <c r="S127" s="16" t="str">
         <f aca="false">IF(AND(G127&lt;&gt;"",COUNT(J127:N127)=5,OR(ISNUMBER(O127),O127="N/A"),P127&lt;&gt;"",Q127&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="128" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -26833,18 +27105,34 @@
       <c r="I128" s="14" t="s">
         <v>555</v>
       </c>
-      <c r="J128" s="15"/>
-      <c r="K128" s="15"/>
-      <c r="L128" s="15"/>
-      <c r="M128" s="15"/>
-      <c r="N128" s="15"/>
-      <c r="O128" s="15"/>
-      <c r="P128" s="15"/>
-      <c r="Q128" s="15"/>
+      <c r="J128" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="K128" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L128" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M128" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N128" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O128" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="P128" s="15" t="s">
+        <v>116</v>
+      </c>
+      <c r="Q128" s="15" t="s">
+        <v>117</v>
+      </c>
       <c r="R128" s="15"/>
       <c r="S128" s="16" t="str">
         <f aca="false">IF(AND(G128&lt;&gt;"",COUNT(J128:N128)=5,OR(ISNUMBER(O128),O128="N/A"),P128&lt;&gt;"",Q128&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="129" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -26875,18 +27163,34 @@
       <c r="I129" s="14" t="s">
         <v>559</v>
       </c>
-      <c r="J129" s="15"/>
-      <c r="K129" s="15"/>
-      <c r="L129" s="15"/>
-      <c r="M129" s="15"/>
-      <c r="N129" s="15"/>
-      <c r="O129" s="15"/>
-      <c r="P129" s="15"/>
-      <c r="Q129" s="15"/>
+      <c r="J129" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="K129" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L129" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M129" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N129" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O129" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="P129" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q129" s="15" t="s">
+        <v>36</v>
+      </c>
       <c r="R129" s="15"/>
       <c r="S129" s="16" t="str">
         <f aca="false">IF(AND(G129&lt;&gt;"",COUNT(J129:N129)=5,OR(ISNUMBER(O129),O129="N/A"),P129&lt;&gt;"",Q129&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="130" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -26913,18 +27217,34 @@
       </c>
       <c r="H130" s="14"/>
       <c r="I130" s="14"/>
-      <c r="J130" s="15"/>
-      <c r="K130" s="15"/>
-      <c r="L130" s="15"/>
-      <c r="M130" s="15"/>
-      <c r="N130" s="15"/>
-      <c r="O130" s="15"/>
-      <c r="P130" s="15"/>
-      <c r="Q130" s="15"/>
+      <c r="J130" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="K130" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L130" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M130" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N130" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O130" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="P130" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q130" s="15" t="s">
+        <v>36</v>
+      </c>
       <c r="R130" s="15"/>
       <c r="S130" s="16" t="str">
         <f aca="false">IF(AND(G130&lt;&gt;"",COUNT(J130:N130)=5,OR(ISNUMBER(O130),O130="N/A"),P130&lt;&gt;"",Q130&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="131" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -26955,18 +27275,34 @@
       <c r="I131" s="14" t="s">
         <v>565</v>
       </c>
-      <c r="J131" s="15"/>
-      <c r="K131" s="15"/>
-      <c r="L131" s="15"/>
-      <c r="M131" s="15"/>
-      <c r="N131" s="15"/>
-      <c r="O131" s="15"/>
-      <c r="P131" s="15"/>
-      <c r="Q131" s="15"/>
+      <c r="J131" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="K131" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L131" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M131" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N131" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O131" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="P131" s="15" t="s">
+        <v>95</v>
+      </c>
+      <c r="Q131" s="15" t="s">
+        <v>36</v>
+      </c>
       <c r="R131" s="15"/>
       <c r="S131" s="16" t="str">
         <f aca="false">IF(AND(G131&lt;&gt;"",COUNT(J131:N131)=5,OR(ISNUMBER(O131),O131="N/A"),P131&lt;&gt;"",Q131&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="132" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -26997,18 +27333,34 @@
       <c r="I132" s="14" t="s">
         <v>569</v>
       </c>
-      <c r="J132" s="15"/>
-      <c r="K132" s="15"/>
-      <c r="L132" s="15"/>
-      <c r="M132" s="15"/>
-      <c r="N132" s="15"/>
-      <c r="O132" s="15"/>
-      <c r="P132" s="15"/>
-      <c r="Q132" s="15"/>
+      <c r="J132" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="K132" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L132" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M132" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N132" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O132" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="P132" s="15" t="s">
+        <v>95</v>
+      </c>
+      <c r="Q132" s="15" t="s">
+        <v>36</v>
+      </c>
       <c r="R132" s="15"/>
       <c r="S132" s="16" t="str">
         <f aca="false">IF(AND(G132&lt;&gt;"",COUNT(J132:N132)=5,OR(ISNUMBER(O132),O132="N/A"),P132&lt;&gt;"",Q132&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="133" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -27039,18 +27391,34 @@
       <c r="I133" s="14" t="s">
         <v>573</v>
       </c>
-      <c r="J133" s="15"/>
-      <c r="K133" s="15"/>
-      <c r="L133" s="15"/>
-      <c r="M133" s="15"/>
-      <c r="N133" s="15"/>
-      <c r="O133" s="15"/>
-      <c r="P133" s="15"/>
-      <c r="Q133" s="15"/>
+      <c r="J133" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="K133" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L133" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M133" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N133" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O133" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="P133" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q133" s="15" t="s">
+        <v>36</v>
+      </c>
       <c r="R133" s="15"/>
       <c r="S133" s="16" t="str">
         <f aca="false">IF(AND(G133&lt;&gt;"",COUNT(J133:N133)=5,OR(ISNUMBER(O133),O133="N/A"),P133&lt;&gt;"",Q133&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="134" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -27081,18 +27449,34 @@
       <c r="I134" s="14" t="s">
         <v>577</v>
       </c>
-      <c r="J134" s="15"/>
-      <c r="K134" s="15"/>
-      <c r="L134" s="15"/>
-      <c r="M134" s="15"/>
-      <c r="N134" s="15"/>
-      <c r="O134" s="15"/>
-      <c r="P134" s="15"/>
-      <c r="Q134" s="15"/>
+      <c r="J134" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="K134" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L134" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M134" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N134" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O134" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="P134" s="15" t="s">
+        <v>116</v>
+      </c>
+      <c r="Q134" s="15" t="s">
+        <v>117</v>
+      </c>
       <c r="R134" s="15"/>
       <c r="S134" s="16" t="str">
         <f aca="false">IF(AND(G134&lt;&gt;"",COUNT(J134:N134)=5,OR(ISNUMBER(O134),O134="N/A"),P134&lt;&gt;"",Q134&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="135" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -27123,18 +27507,34 @@
       <c r="I135" s="14" t="s">
         <v>581</v>
       </c>
-      <c r="J135" s="15"/>
-      <c r="K135" s="15"/>
-      <c r="L135" s="15"/>
-      <c r="M135" s="15"/>
-      <c r="N135" s="15"/>
-      <c r="O135" s="15"/>
-      <c r="P135" s="15"/>
-      <c r="Q135" s="15"/>
+      <c r="J135" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="K135" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L135" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M135" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N135" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O135" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="P135" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q135" s="15" t="s">
+        <v>36</v>
+      </c>
       <c r="R135" s="15"/>
       <c r="S135" s="16" t="str">
         <f aca="false">IF(AND(G135&lt;&gt;"",COUNT(J135:N135)=5,OR(ISNUMBER(O135),O135="N/A"),P135&lt;&gt;"",Q135&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="136" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -27161,18 +27561,34 @@
       </c>
       <c r="H136" s="14"/>
       <c r="I136" s="14"/>
-      <c r="J136" s="15"/>
-      <c r="K136" s="15"/>
-      <c r="L136" s="15"/>
-      <c r="M136" s="15"/>
-      <c r="N136" s="15"/>
-      <c r="O136" s="15"/>
-      <c r="P136" s="15"/>
-      <c r="Q136" s="15"/>
+      <c r="J136" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="K136" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L136" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M136" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N136" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="O136" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="P136" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q136" s="15" t="s">
+        <v>36</v>
+      </c>
       <c r="R136" s="15"/>
       <c r="S136" s="16" t="str">
         <f aca="false">IF(AND(G136&lt;&gt;"",COUNT(J136:N136)=5,OR(ISNUMBER(O136),O136="N/A"),P136&lt;&gt;"",Q136&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="137" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -27203,18 +27619,34 @@
       <c r="I137" s="14" t="s">
         <v>587</v>
       </c>
-      <c r="J137" s="15"/>
-      <c r="K137" s="15"/>
-      <c r="L137" s="15"/>
-      <c r="M137" s="15"/>
-      <c r="N137" s="15"/>
-      <c r="O137" s="15"/>
-      <c r="P137" s="15"/>
-      <c r="Q137" s="15"/>
+      <c r="J137" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="K137" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L137" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M137" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N137" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O137" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="P137" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q137" s="15" t="s">
+        <v>36</v>
+      </c>
       <c r="R137" s="15"/>
       <c r="S137" s="16" t="str">
         <f aca="false">IF(AND(G137&lt;&gt;"",COUNT(J137:N137)=5,OR(ISNUMBER(O137),O137="N/A"),P137&lt;&gt;"",Q137&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="138" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -27245,18 +27677,34 @@
       <c r="I138" s="14" t="s">
         <v>591</v>
       </c>
-      <c r="J138" s="15"/>
-      <c r="K138" s="15"/>
-      <c r="L138" s="15"/>
-      <c r="M138" s="15"/>
-      <c r="N138" s="15"/>
-      <c r="O138" s="15"/>
-      <c r="P138" s="15"/>
-      <c r="Q138" s="15"/>
+      <c r="J138" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="K138" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L138" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M138" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N138" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O138" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="P138" s="15" t="s">
+        <v>116</v>
+      </c>
+      <c r="Q138" s="15" t="s">
+        <v>117</v>
+      </c>
       <c r="R138" s="15"/>
       <c r="S138" s="16" t="str">
         <f aca="false">IF(AND(G138&lt;&gt;"",COUNT(J138:N138)=5,OR(ISNUMBER(O138),O138="N/A"),P138&lt;&gt;"",Q138&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="139" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -27287,18 +27735,34 @@
       <c r="I139" s="14" t="s">
         <v>595</v>
       </c>
-      <c r="J139" s="15"/>
-      <c r="K139" s="15"/>
-      <c r="L139" s="15"/>
-      <c r="M139" s="15"/>
-      <c r="N139" s="15"/>
-      <c r="O139" s="15"/>
-      <c r="P139" s="15"/>
-      <c r="Q139" s="15"/>
+      <c r="J139" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="K139" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="L139" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M139" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N139" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O139" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="P139" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q139" s="15" t="s">
+        <v>75</v>
+      </c>
       <c r="R139" s="15"/>
       <c r="S139" s="16" t="str">
         <f aca="false">IF(AND(G139&lt;&gt;"",COUNT(J139:N139)=5,OR(ISNUMBER(O139),O139="N/A"),P139&lt;&gt;"",Q139&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="140" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -27325,18 +27789,34 @@
       </c>
       <c r="H140" s="14"/>
       <c r="I140" s="14"/>
-      <c r="J140" s="15"/>
-      <c r="K140" s="15"/>
-      <c r="L140" s="15"/>
-      <c r="M140" s="15"/>
-      <c r="N140" s="15"/>
-      <c r="O140" s="15"/>
-      <c r="P140" s="15"/>
-      <c r="Q140" s="15"/>
+      <c r="J140" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="K140" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L140" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M140" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N140" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O140" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="P140" s="15" t="s">
+        <v>95</v>
+      </c>
+      <c r="Q140" s="15" t="s">
+        <v>36</v>
+      </c>
       <c r="R140" s="15"/>
       <c r="S140" s="16" t="str">
         <f aca="false">IF(AND(G140&lt;&gt;"",COUNT(J140:N140)=5,OR(ISNUMBER(O140),O140="N/A"),P140&lt;&gt;"",Q140&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="141" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -27363,18 +27843,34 @@
       </c>
       <c r="H141" s="14"/>
       <c r="I141" s="14"/>
-      <c r="J141" s="15"/>
-      <c r="K141" s="15"/>
-      <c r="L141" s="15"/>
-      <c r="M141" s="15"/>
-      <c r="N141" s="15"/>
-      <c r="O141" s="15"/>
-      <c r="P141" s="15"/>
-      <c r="Q141" s="15"/>
+      <c r="J141" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="K141" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L141" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M141" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N141" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O141" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="P141" s="15" t="s">
+        <v>116</v>
+      </c>
+      <c r="Q141" s="15" t="s">
+        <v>117</v>
+      </c>
       <c r="R141" s="15"/>
       <c r="S141" s="16" t="str">
         <f aca="false">IF(AND(G141&lt;&gt;"",COUNT(J141:N141)=5,OR(ISNUMBER(O141),O141="N/A"),P141&lt;&gt;"",Q141&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="142" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -27405,18 +27901,34 @@
       <c r="I142" s="14" t="s">
         <v>603</v>
       </c>
-      <c r="J142" s="15"/>
-      <c r="K142" s="15"/>
-      <c r="L142" s="15"/>
-      <c r="M142" s="15"/>
-      <c r="N142" s="15"/>
-      <c r="O142" s="15"/>
-      <c r="P142" s="15"/>
-      <c r="Q142" s="15"/>
+      <c r="J142" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="K142" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L142" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M142" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N142" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O142" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="P142" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q142" s="15" t="s">
+        <v>75</v>
+      </c>
       <c r="R142" s="15"/>
       <c r="S142" s="16" t="str">
         <f aca="false">IF(AND(G142&lt;&gt;"",COUNT(J142:N142)=5,OR(ISNUMBER(O142),O142="N/A"),P142&lt;&gt;"",Q142&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="143" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -27447,18 +27959,34 @@
       <c r="I143" s="14" t="s">
         <v>606</v>
       </c>
-      <c r="J143" s="15"/>
-      <c r="K143" s="15"/>
-      <c r="L143" s="15"/>
-      <c r="M143" s="15"/>
-      <c r="N143" s="15"/>
-      <c r="O143" s="15"/>
-      <c r="P143" s="15"/>
-      <c r="Q143" s="15"/>
+      <c r="J143" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="K143" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L143" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M143" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N143" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O143" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="P143" s="15" t="s">
+        <v>116</v>
+      </c>
+      <c r="Q143" s="15" t="s">
+        <v>117</v>
+      </c>
       <c r="R143" s="15"/>
       <c r="S143" s="16" t="str">
         <f aca="false">IF(AND(G143&lt;&gt;"",COUNT(J143:N143)=5,OR(ISNUMBER(O143),O143="N/A"),P143&lt;&gt;"",Q143&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="144" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -27489,18 +28017,34 @@
       <c r="I144" s="14" t="s">
         <v>610</v>
       </c>
-      <c r="J144" s="15"/>
-      <c r="K144" s="15"/>
-      <c r="L144" s="15"/>
-      <c r="M144" s="15"/>
-      <c r="N144" s="15"/>
-      <c r="O144" s="15"/>
-      <c r="P144" s="15"/>
-      <c r="Q144" s="15"/>
+      <c r="J144" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="K144" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L144" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M144" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N144" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O144" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="P144" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q144" s="15" t="s">
+        <v>36</v>
+      </c>
       <c r="R144" s="15"/>
       <c r="S144" s="16" t="str">
         <f aca="false">IF(AND(G144&lt;&gt;"",COUNT(J144:N144)=5,OR(ISNUMBER(O144),O144="N/A"),P144&lt;&gt;"",Q144&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="145" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
[HUMAN-VALIDATION]: completed human test cases validation.
</commit_message>
<xml_diff>
--- a/thesis_evidence/validazione_umana/02_VALUTAZIONE_UMANA.xlsx
+++ b/thesis_evidence/validazione_umana/02_VALUTAZIONE_UMANA.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3353" uniqueCount="1071">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3413" uniqueCount="1071">
   <si>
     <t xml:space="preserve">Valutazione delle 250 risposte del test</t>
   </si>
@@ -20207,7 +20207,7 @@
       </c>
       <c r="B7" s="9" t="n">
         <f aca="false">COUNTIF(S9:S258,"OK")</f>
-        <v>223</v>
+        <v>250</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -33057,18 +33057,34 @@
       <c r="I232" s="14" t="s">
         <v>926</v>
       </c>
-      <c r="J232" s="15"/>
-      <c r="K232" s="15"/>
-      <c r="L232" s="15"/>
-      <c r="M232" s="15"/>
-      <c r="N232" s="15"/>
-      <c r="O232" s="15"/>
-      <c r="P232" s="15"/>
-      <c r="Q232" s="15"/>
+      <c r="J232" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="K232" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L232" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M232" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N232" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O232" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="P232" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q232" s="15" t="s">
+        <v>75</v>
+      </c>
       <c r="R232" s="15"/>
       <c r="S232" s="16" t="str">
         <f aca="false">IF(AND(G232&lt;&gt;"",COUNT(J232:N232)=5,OR(ISNUMBER(O232),O232="N/A"),P232&lt;&gt;"",Q232&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="233" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -33099,18 +33115,34 @@
       <c r="I233" s="14" t="s">
         <v>930</v>
       </c>
-      <c r="J233" s="15"/>
-      <c r="K233" s="15"/>
-      <c r="L233" s="15"/>
-      <c r="M233" s="15"/>
-      <c r="N233" s="15"/>
-      <c r="O233" s="15"/>
-      <c r="P233" s="15"/>
-      <c r="Q233" s="15"/>
+      <c r="J233" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="K233" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L233" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M233" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N233" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O233" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="P233" s="15" t="s">
+        <v>116</v>
+      </c>
+      <c r="Q233" s="15" t="s">
+        <v>117</v>
+      </c>
       <c r="R233" s="15"/>
       <c r="S233" s="16" t="str">
         <f aca="false">IF(AND(G233&lt;&gt;"",COUNT(J233:N233)=5,OR(ISNUMBER(O233),O233="N/A"),P233&lt;&gt;"",Q233&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="234" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -33137,18 +33169,34 @@
       </c>
       <c r="H234" s="14"/>
       <c r="I234" s="14"/>
-      <c r="J234" s="15"/>
-      <c r="K234" s="15"/>
-      <c r="L234" s="15"/>
-      <c r="M234" s="15"/>
-      <c r="N234" s="15"/>
-      <c r="O234" s="15"/>
-      <c r="P234" s="15"/>
-      <c r="Q234" s="15"/>
+      <c r="J234" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="K234" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L234" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M234" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N234" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O234" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="P234" s="15" t="s">
+        <v>95</v>
+      </c>
+      <c r="Q234" s="15" t="s">
+        <v>36</v>
+      </c>
       <c r="R234" s="15"/>
       <c r="S234" s="16" t="str">
         <f aca="false">IF(AND(G234&lt;&gt;"",COUNT(J234:N234)=5,OR(ISNUMBER(O234),O234="N/A"),P234&lt;&gt;"",Q234&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="235" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -33179,18 +33227,34 @@
       <c r="I235" s="14" t="s">
         <v>936</v>
       </c>
-      <c r="J235" s="15"/>
-      <c r="K235" s="15"/>
-      <c r="L235" s="15"/>
-      <c r="M235" s="15"/>
-      <c r="N235" s="15"/>
-      <c r="O235" s="15"/>
-      <c r="P235" s="15"/>
-      <c r="Q235" s="15"/>
+      <c r="J235" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="K235" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L235" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M235" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N235" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O235" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="P235" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q235" s="15" t="s">
+        <v>36</v>
+      </c>
       <c r="R235" s="15"/>
       <c r="S235" s="16" t="str">
         <f aca="false">IF(AND(G235&lt;&gt;"",COUNT(J235:N235)=5,OR(ISNUMBER(O235),O235="N/A"),P235&lt;&gt;"",Q235&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="236" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -33221,18 +33285,34 @@
       <c r="I236" s="14" t="s">
         <v>940</v>
       </c>
-      <c r="J236" s="15"/>
-      <c r="K236" s="15"/>
-      <c r="L236" s="15"/>
-      <c r="M236" s="15"/>
-      <c r="N236" s="15"/>
-      <c r="O236" s="15"/>
-      <c r="P236" s="15"/>
-      <c r="Q236" s="15"/>
+      <c r="J236" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="K236" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L236" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M236" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N236" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O236" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="P236" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q236" s="15" t="s">
+        <v>36</v>
+      </c>
       <c r="R236" s="15"/>
       <c r="S236" s="16" t="str">
         <f aca="false">IF(AND(G236&lt;&gt;"",COUNT(J236:N236)=5,OR(ISNUMBER(O236),O236="N/A"),P236&lt;&gt;"",Q236&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="237" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -33263,18 +33343,34 @@
       <c r="I237" s="14" t="s">
         <v>944</v>
       </c>
-      <c r="J237" s="15"/>
-      <c r="K237" s="15"/>
-      <c r="L237" s="15"/>
-      <c r="M237" s="15"/>
-      <c r="N237" s="15"/>
-      <c r="O237" s="15"/>
-      <c r="P237" s="15"/>
-      <c r="Q237" s="15"/>
+      <c r="J237" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="K237" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L237" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M237" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N237" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O237" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="P237" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q237" s="15" t="s">
+        <v>36</v>
+      </c>
       <c r="R237" s="15"/>
       <c r="S237" s="16" t="str">
         <f aca="false">IF(AND(G237&lt;&gt;"",COUNT(J237:N237)=5,OR(ISNUMBER(O237),O237="N/A"),P237&lt;&gt;"",Q237&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="238" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -33301,18 +33397,34 @@
       </c>
       <c r="H238" s="14"/>
       <c r="I238" s="14"/>
-      <c r="J238" s="15"/>
-      <c r="K238" s="15"/>
-      <c r="L238" s="15"/>
-      <c r="M238" s="15"/>
-      <c r="N238" s="15"/>
-      <c r="O238" s="15"/>
-      <c r="P238" s="15"/>
-      <c r="Q238" s="15"/>
+      <c r="J238" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="K238" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L238" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M238" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N238" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O238" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="P238" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q238" s="15" t="s">
+        <v>125</v>
+      </c>
       <c r="R238" s="15"/>
       <c r="S238" s="16" t="str">
         <f aca="false">IF(AND(G238&lt;&gt;"",COUNT(J238:N238)=5,OR(ISNUMBER(O238),O238="N/A"),P238&lt;&gt;"",Q238&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="239" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -33343,18 +33455,34 @@
       <c r="I239" s="14" t="s">
         <v>950</v>
       </c>
-      <c r="J239" s="15"/>
-      <c r="K239" s="15"/>
-      <c r="L239" s="15"/>
-      <c r="M239" s="15"/>
-      <c r="N239" s="15"/>
-      <c r="O239" s="15"/>
-      <c r="P239" s="15"/>
-      <c r="Q239" s="15"/>
+      <c r="J239" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="K239" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L239" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M239" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N239" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O239" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="P239" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q239" s="15" t="s">
+        <v>36</v>
+      </c>
       <c r="R239" s="15"/>
       <c r="S239" s="16" t="str">
         <f aca="false">IF(AND(G239&lt;&gt;"",COUNT(J239:N239)=5,OR(ISNUMBER(O239),O239="N/A"),P239&lt;&gt;"",Q239&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="240" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -33385,18 +33513,34 @@
       <c r="I240" s="14" t="s">
         <v>954</v>
       </c>
-      <c r="J240" s="15"/>
-      <c r="K240" s="15"/>
-      <c r="L240" s="15"/>
-      <c r="M240" s="15"/>
-      <c r="N240" s="15"/>
-      <c r="O240" s="15"/>
-      <c r="P240" s="15"/>
-      <c r="Q240" s="15"/>
+      <c r="J240" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="K240" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L240" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M240" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N240" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O240" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="P240" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q240" s="15" t="s">
+        <v>36</v>
+      </c>
       <c r="R240" s="15"/>
       <c r="S240" s="16" t="str">
         <f aca="false">IF(AND(G240&lt;&gt;"",COUNT(J240:N240)=5,OR(ISNUMBER(O240),O240="N/A"),P240&lt;&gt;"",Q240&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="241" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -33427,18 +33571,34 @@
       <c r="I241" s="14" t="s">
         <v>958</v>
       </c>
-      <c r="J241" s="15"/>
-      <c r="K241" s="15"/>
-      <c r="L241" s="15"/>
-      <c r="M241" s="15"/>
-      <c r="N241" s="15"/>
-      <c r="O241" s="15"/>
-      <c r="P241" s="15"/>
-      <c r="Q241" s="15"/>
+      <c r="J241" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="K241" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L241" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M241" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N241" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O241" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="P241" s="15" t="s">
+        <v>95</v>
+      </c>
+      <c r="Q241" s="15" t="s">
+        <v>36</v>
+      </c>
       <c r="R241" s="15"/>
       <c r="S241" s="16" t="str">
         <f aca="false">IF(AND(G241&lt;&gt;"",COUNT(J241:N241)=5,OR(ISNUMBER(O241),O241="N/A"),P241&lt;&gt;"",Q241&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="242" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -33469,18 +33629,34 @@
       <c r="I242" s="14" t="s">
         <v>962</v>
       </c>
-      <c r="J242" s="15"/>
-      <c r="K242" s="15"/>
-      <c r="L242" s="15"/>
-      <c r="M242" s="15"/>
-      <c r="N242" s="15"/>
-      <c r="O242" s="15"/>
-      <c r="P242" s="15"/>
-      <c r="Q242" s="15"/>
+      <c r="J242" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="K242" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L242" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M242" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N242" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O242" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="P242" s="15" t="s">
+        <v>95</v>
+      </c>
+      <c r="Q242" s="15" t="s">
+        <v>75</v>
+      </c>
       <c r="R242" s="15"/>
       <c r="S242" s="16" t="str">
         <f aca="false">IF(AND(G242&lt;&gt;"",COUNT(J242:N242)=5,OR(ISNUMBER(O242),O242="N/A"),P242&lt;&gt;"",Q242&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="243" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -33511,18 +33687,34 @@
       <c r="I243" s="14" t="s">
         <v>966</v>
       </c>
-      <c r="J243" s="15"/>
-      <c r="K243" s="15"/>
-      <c r="L243" s="15"/>
-      <c r="M243" s="15"/>
-      <c r="N243" s="15"/>
-      <c r="O243" s="15"/>
-      <c r="P243" s="15"/>
-      <c r="Q243" s="15"/>
+      <c r="J243" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="K243" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L243" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M243" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N243" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O243" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="P243" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q243" s="15" t="s">
+        <v>36</v>
+      </c>
       <c r="R243" s="15"/>
       <c r="S243" s="16" t="str">
         <f aca="false">IF(AND(G243&lt;&gt;"",COUNT(J243:N243)=5,OR(ISNUMBER(O243),O243="N/A"),P243&lt;&gt;"",Q243&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="244" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -33549,18 +33741,34 @@
       </c>
       <c r="H244" s="14"/>
       <c r="I244" s="14"/>
-      <c r="J244" s="15"/>
-      <c r="K244" s="15"/>
-      <c r="L244" s="15"/>
-      <c r="M244" s="15"/>
-      <c r="N244" s="15"/>
-      <c r="O244" s="15"/>
-      <c r="P244" s="15"/>
-      <c r="Q244" s="15"/>
+      <c r="J244" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="K244" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L244" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M244" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N244" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O244" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="P244" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q244" s="15" t="s">
+        <v>125</v>
+      </c>
       <c r="R244" s="15"/>
       <c r="S244" s="16" t="str">
         <f aca="false">IF(AND(G244&lt;&gt;"",COUNT(J244:N244)=5,OR(ISNUMBER(O244),O244="N/A"),P244&lt;&gt;"",Q244&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="245" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -33587,18 +33795,34 @@
       </c>
       <c r="H245" s="14"/>
       <c r="I245" s="14"/>
-      <c r="J245" s="15"/>
-      <c r="K245" s="15"/>
-      <c r="L245" s="15"/>
-      <c r="M245" s="15"/>
-      <c r="N245" s="15"/>
-      <c r="O245" s="15"/>
-      <c r="P245" s="15"/>
-      <c r="Q245" s="15"/>
+      <c r="J245" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="K245" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L245" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M245" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N245" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O245" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="P245" s="15" t="s">
+        <v>95</v>
+      </c>
+      <c r="Q245" s="15" t="s">
+        <v>36</v>
+      </c>
       <c r="R245" s="15"/>
       <c r="S245" s="16" t="str">
         <f aca="false">IF(AND(G245&lt;&gt;"",COUNT(J245:N245)=5,OR(ISNUMBER(O245),O245="N/A"),P245&lt;&gt;"",Q245&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="246" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -33629,18 +33853,34 @@
       <c r="I246" s="14" t="s">
         <v>974</v>
       </c>
-      <c r="J246" s="15"/>
-      <c r="K246" s="15"/>
-      <c r="L246" s="15"/>
-      <c r="M246" s="15"/>
-      <c r="N246" s="15"/>
-      <c r="O246" s="15"/>
-      <c r="P246" s="15"/>
-      <c r="Q246" s="15"/>
+      <c r="J246" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="K246" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L246" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M246" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N246" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O246" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="P246" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q246" s="15" t="s">
+        <v>36</v>
+      </c>
       <c r="R246" s="15"/>
       <c r="S246" s="16" t="str">
         <f aca="false">IF(AND(G246&lt;&gt;"",COUNT(J246:N246)=5,OR(ISNUMBER(O246),O246="N/A"),P246&lt;&gt;"",Q246&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="247" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -33667,18 +33907,34 @@
       </c>
       <c r="H247" s="14"/>
       <c r="I247" s="14"/>
-      <c r="J247" s="15"/>
-      <c r="K247" s="15"/>
-      <c r="L247" s="15"/>
-      <c r="M247" s="15"/>
-      <c r="N247" s="15"/>
-      <c r="O247" s="15"/>
-      <c r="P247" s="15"/>
-      <c r="Q247" s="15"/>
+      <c r="J247" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="K247" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L247" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M247" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N247" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O247" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="P247" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q247" s="15" t="s">
+        <v>125</v>
+      </c>
       <c r="R247" s="15"/>
       <c r="S247" s="16" t="str">
         <f aca="false">IF(AND(G247&lt;&gt;"",COUNT(J247:N247)=5,OR(ISNUMBER(O247),O247="N/A"),P247&lt;&gt;"",Q247&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="248" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -33705,18 +33961,34 @@
       </c>
       <c r="H248" s="14"/>
       <c r="I248" s="14"/>
-      <c r="J248" s="15"/>
-      <c r="K248" s="15"/>
-      <c r="L248" s="15"/>
-      <c r="M248" s="15"/>
-      <c r="N248" s="15"/>
-      <c r="O248" s="15"/>
-      <c r="P248" s="15"/>
-      <c r="Q248" s="15"/>
+      <c r="J248" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="K248" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L248" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M248" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N248" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O248" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="P248" s="15" t="s">
+        <v>74</v>
+      </c>
+      <c r="Q248" s="15" t="s">
+        <v>104</v>
+      </c>
       <c r="R248" s="15"/>
       <c r="S248" s="16" t="str">
         <f aca="false">IF(AND(G248&lt;&gt;"",COUNT(J248:N248)=5,OR(ISNUMBER(O248),O248="N/A"),P248&lt;&gt;"",Q248&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="249" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -33747,18 +34019,34 @@
       <c r="I249" s="14" t="s">
         <v>982</v>
       </c>
-      <c r="J249" s="15"/>
-      <c r="K249" s="15"/>
-      <c r="L249" s="15"/>
-      <c r="M249" s="15"/>
-      <c r="N249" s="15"/>
-      <c r="O249" s="15"/>
-      <c r="P249" s="15"/>
-      <c r="Q249" s="15"/>
+      <c r="J249" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="K249" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L249" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M249" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N249" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="O249" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="P249" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q249" s="15" t="s">
+        <v>36</v>
+      </c>
       <c r="R249" s="15"/>
       <c r="S249" s="16" t="str">
         <f aca="false">IF(AND(G249&lt;&gt;"",COUNT(J249:N249)=5,OR(ISNUMBER(O249),O249="N/A"),P249&lt;&gt;"",Q249&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="250" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -33789,18 +34077,34 @@
       <c r="I250" s="14" t="s">
         <v>986</v>
       </c>
-      <c r="J250" s="15"/>
-      <c r="K250" s="15"/>
-      <c r="L250" s="15"/>
-      <c r="M250" s="15"/>
-      <c r="N250" s="15"/>
-      <c r="O250" s="15"/>
-      <c r="P250" s="15"/>
-      <c r="Q250" s="15"/>
+      <c r="J250" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="K250" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L250" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M250" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N250" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O250" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="P250" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q250" s="15" t="s">
+        <v>36</v>
+      </c>
       <c r="R250" s="15"/>
       <c r="S250" s="16" t="str">
         <f aca="false">IF(AND(G250&lt;&gt;"",COUNT(J250:N250)=5,OR(ISNUMBER(O250),O250="N/A"),P250&lt;&gt;"",Q250&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="251" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -33831,18 +34135,34 @@
       <c r="I251" s="14" t="s">
         <v>990</v>
       </c>
-      <c r="J251" s="15"/>
-      <c r="K251" s="15"/>
-      <c r="L251" s="15"/>
-      <c r="M251" s="15"/>
-      <c r="N251" s="15"/>
-      <c r="O251" s="15"/>
-      <c r="P251" s="15"/>
-      <c r="Q251" s="15"/>
+      <c r="J251" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="K251" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L251" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M251" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N251" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O251" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="P251" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q251" s="15" t="s">
+        <v>36</v>
+      </c>
       <c r="R251" s="15"/>
       <c r="S251" s="16" t="str">
         <f aca="false">IF(AND(G251&lt;&gt;"",COUNT(J251:N251)=5,OR(ISNUMBER(O251),O251="N/A"),P251&lt;&gt;"",Q251&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="252" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -33873,18 +34193,34 @@
       <c r="I252" s="14" t="s">
         <v>994</v>
       </c>
-      <c r="J252" s="15"/>
-      <c r="K252" s="15"/>
-      <c r="L252" s="15"/>
-      <c r="M252" s="15"/>
-      <c r="N252" s="15"/>
-      <c r="O252" s="15"/>
-      <c r="P252" s="15"/>
-      <c r="Q252" s="15"/>
+      <c r="J252" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="K252" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L252" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M252" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N252" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O252" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="P252" s="15" t="s">
+        <v>95</v>
+      </c>
+      <c r="Q252" s="15" t="s">
+        <v>75</v>
+      </c>
       <c r="R252" s="15"/>
       <c r="S252" s="16" t="str">
         <f aca="false">IF(AND(G252&lt;&gt;"",COUNT(J252:N252)=5,OR(ISNUMBER(O252),O252="N/A"),P252&lt;&gt;"",Q252&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="253" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -33915,18 +34251,34 @@
       <c r="I253" s="14" t="s">
         <v>998</v>
       </c>
-      <c r="J253" s="15"/>
-      <c r="K253" s="15"/>
-      <c r="L253" s="15"/>
-      <c r="M253" s="15"/>
-      <c r="N253" s="15"/>
-      <c r="O253" s="15"/>
-      <c r="P253" s="15"/>
-      <c r="Q253" s="15"/>
+      <c r="J253" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="K253" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L253" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M253" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N253" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O253" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="P253" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q253" s="15" t="s">
+        <v>36</v>
+      </c>
       <c r="R253" s="15"/>
       <c r="S253" s="16" t="str">
         <f aca="false">IF(AND(G253&lt;&gt;"",COUNT(J253:N253)=5,OR(ISNUMBER(O253),O253="N/A"),P253&lt;&gt;"",Q253&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="254" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -33957,18 +34309,34 @@
       <c r="I254" s="14" t="s">
         <v>1002</v>
       </c>
-      <c r="J254" s="15"/>
-      <c r="K254" s="15"/>
-      <c r="L254" s="15"/>
-      <c r="M254" s="15"/>
-      <c r="N254" s="15"/>
-      <c r="O254" s="15"/>
-      <c r="P254" s="15"/>
-      <c r="Q254" s="15"/>
+      <c r="J254" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="K254" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L254" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M254" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N254" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O254" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="P254" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q254" s="15" t="s">
+        <v>36</v>
+      </c>
       <c r="R254" s="15"/>
       <c r="S254" s="16" t="str">
         <f aca="false">IF(AND(G254&lt;&gt;"",COUNT(J254:N254)=5,OR(ISNUMBER(O254),O254="N/A"),P254&lt;&gt;"",Q254&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="255" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -33999,18 +34367,34 @@
       <c r="I255" s="14" t="s">
         <v>1006</v>
       </c>
-      <c r="J255" s="15"/>
-      <c r="K255" s="15"/>
-      <c r="L255" s="15"/>
-      <c r="M255" s="15"/>
-      <c r="N255" s="15"/>
-      <c r="O255" s="15"/>
-      <c r="P255" s="15"/>
-      <c r="Q255" s="15"/>
+      <c r="J255" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="K255" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L255" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M255" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N255" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O255" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="P255" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q255" s="15" t="s">
+        <v>36</v>
+      </c>
       <c r="R255" s="15"/>
       <c r="S255" s="16" t="str">
         <f aca="false">IF(AND(G255&lt;&gt;"",COUNT(J255:N255)=5,OR(ISNUMBER(O255),O255="N/A"),P255&lt;&gt;"",Q255&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="256" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -34041,18 +34425,34 @@
       <c r="I256" s="14" t="s">
         <v>1010</v>
       </c>
-      <c r="J256" s="15"/>
-      <c r="K256" s="15"/>
-      <c r="L256" s="15"/>
-      <c r="M256" s="15"/>
-      <c r="N256" s="15"/>
-      <c r="O256" s="15"/>
-      <c r="P256" s="15"/>
-      <c r="Q256" s="15"/>
+      <c r="J256" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="K256" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L256" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M256" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N256" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O256" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="P256" s="15" t="s">
+        <v>95</v>
+      </c>
+      <c r="Q256" s="15" t="s">
+        <v>36</v>
+      </c>
       <c r="R256" s="15"/>
       <c r="S256" s="16" t="str">
         <f aca="false">IF(AND(G256&lt;&gt;"",COUNT(J256:N256)=5,OR(ISNUMBER(O256),O256="N/A"),P256&lt;&gt;"",Q256&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="257" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -34083,18 +34483,34 @@
       <c r="I257" s="14" t="s">
         <v>1014</v>
       </c>
-      <c r="J257" s="15"/>
-      <c r="K257" s="15"/>
-      <c r="L257" s="15"/>
-      <c r="M257" s="15"/>
-      <c r="N257" s="15"/>
-      <c r="O257" s="15"/>
-      <c r="P257" s="15"/>
-      <c r="Q257" s="15"/>
+      <c r="J257" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="K257" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L257" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M257" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N257" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O257" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="P257" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q257" s="15" t="s">
+        <v>36</v>
+      </c>
       <c r="R257" s="15"/>
       <c r="S257" s="16" t="str">
         <f aca="false">IF(AND(G257&lt;&gt;"",COUNT(J257:N257)=5,OR(ISNUMBER(O257),O257="N/A"),P257&lt;&gt;"",Q257&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="258" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -34125,18 +34541,34 @@
       <c r="I258" s="14" t="s">
         <v>1017</v>
       </c>
-      <c r="J258" s="15"/>
-      <c r="K258" s="15"/>
-      <c r="L258" s="15"/>
-      <c r="M258" s="15"/>
-      <c r="N258" s="15"/>
-      <c r="O258" s="15"/>
-      <c r="P258" s="15"/>
-      <c r="Q258" s="15"/>
+      <c r="J258" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="K258" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L258" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M258" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N258" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O258" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="P258" s="15" t="s">
+        <v>95</v>
+      </c>
+      <c r="Q258" s="15" t="s">
+        <v>36</v>
+      </c>
       <c r="R258" s="15"/>
       <c r="S258" s="16" t="str">
         <f aca="false">IF(AND(G258&lt;&gt;"",COUNT(J258:N258)=5,OR(ISNUMBER(O258),O258="N/A"),P258&lt;&gt;"",Q258&lt;&gt;""),"OK","DA COMPLETARE")</f>
-        <v>DA COMPLETARE</v>
+        <v>OK</v>
       </c>
     </row>
   </sheetData>
@@ -34152,36 +34584,36 @@
       <formula>NOT(ISERROR(SEARCH("DA COMPLETARE",S9)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="16">
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J9:J81 J111:J258" type="list">
+  <dataValidations count="24">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J9:J81 J111:J231" type="list">
       <formula1>"0,1,2,3"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="K9:K81 K111:K258" type="list">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="K9:K81 K111:K231" type="list">
       <formula1>"0,1,2,3"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="L9:L81 L111:L258" type="list">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="L9:L81 L111:L231" type="list">
       <formula1>"0,1,2,3"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="M9:M81 M111:M258" type="list">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="M9:M81 M111:M231" type="list">
       <formula1>"0,1,2,3"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="N9:N81 N111:N258" type="list">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="N9:N81 N111:N231" type="list">
       <formula1>"0,1,2,3"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="O9:O81 O111:O258" type="list">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="O9:O81 O111:O231" type="list">
       <formula1>"0,1,2,3,N/A"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="P9:P81 P111:P258" type="list">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="P9:P81 P111:P231" type="list">
       <formula1>"CORRETTA,PARZIALMENTE_CORRETTA,ERRATA,NON_INDICATA"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="Q9:Q81 Q111:Q258" type="list">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="Q9:Q81 Q111:Q231" type="list">
       <formula1>"NESSUNO,SOURCE_NOT_RETRIEVED,SOURCE_OUTSIDE_TOP_K,SOURCE_IN_PROMPT_IGNORED,TELEMETRY_MISINTERPRETED,WRONG_ROOT_CAUSE,INVALID_CITATION,UNSUPPORTED_CLAIM,INCOMPLETE_RESPONSE,UNSAFE_ACTION"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -34214,6 +34646,38 @@
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="Q82:Q110" type="list">
+      <formula1>"NESSUNO,SOURCE_NOT_RETRIEVED,SOURCE_OUTSIDE_TOP_K,SOURCE_IN_PROMPT_IGNORED,TELEMETRY_MISINTERPRETED,WRONG_ROOT_CAUSE,INVALID_CITATION,UNSUPPORTED_CLAIM,INCOMPLETE_RESPONSE,UNSAFE_ACTION"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J232:J258" type="list">
+      <formula1>"0,1,2,3"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="K232:K258" type="list">
+      <formula1>"0,1,2,3"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="L232:L258" type="list">
+      <formula1>"0,1,2,3"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="M232:M258" type="list">
+      <formula1>"0,1,2,3"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="N232:N258" type="list">
+      <formula1>"0,1,2,3"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="O232:O258" type="list">
+      <formula1>"0,1,2,3,N/A"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="P232:P258" type="list">
+      <formula1>"CORRETTA,PARZIALMENTE_CORRETTA,ERRATA,NON_INDICATA"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="Q232:Q258" type="list">
       <formula1>"NESSUNO,SOURCE_NOT_RETRIEVED,SOURCE_OUTSIDE_TOP_K,SOURCE_IN_PROMPT_IGNORED,TELEMETRY_MISINTERPRETED,WRONG_ROOT_CAUSE,INVALID_CITATION,UNSUPPORTED_CLAIM,INCOMPLETE_RESPONSE,UNSAFE_ACTION"</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>